<commit_message>
Datenaufbereitung als Skript ergänzt, openpyxl ergänzt, Fehleranalyse aktualisiert
</commit_message>
<xml_diff>
--- a/results/fehleranalyse.xlsx
+++ b/results/fehleranalyse.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>11148</v>
+        <v>2970</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -459,22 +459,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Sichere Verwaltung medizinischer Daten</t>
+          <t>Benötigte Unterstützung bei Abrechnungsproblemen</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Können detaillierte Anleitungen zur Sicherung medizinischer Daten in Microsoft Teams unter Verwendung von Django 3.2 für Krankenhäuser bereitgestellt werden? Es ist entscheidend, dass die Sicherheit und Vertraulichkeit der Patientendaten gewährleistet sind. Bitte geben Sie Anleitungen zur Umsetzung von Sicherheitsmaßnahmen und zur Einhaltung der Vorschriften an.</t>
+          <t>Bei mehreren IT-Produkten eines Gesundheitsdienstleisters treten Abrechnungsprobleme auf. Trotz grundlegender Fehlerbehebung durch Systemneustarts besteht das Problem weiterhin. Ich vermute, dass es auf Integrationsfehler oder veraltete Zahlungs-Module zurückzuführen ist. Bitte schätzen Sie, ob Sie die Angelegenheit zeitnah annehmen und eine Lösung bereitstellen können. Lassen Sie mich bitte wissen, falls Sie weitere Informationen benötigen, um das Problem zu beheben. Ich freue mich auf Ihre Rückmeldung. Vielen Dank für Ihre Unterstützung.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12618</v>
+        <v>11148</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Vertriebsanfrage</t>
+          <t>Rechnung/Zahlung</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -484,18 +484,18 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Datenverlust-Ereignis in Gesundheitsversorgungssystem</t>
+          <t>Sichere Verwaltung medizinischer Daten</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Beim Gesundheitsversorgungssystem ist ein Datensicherheitsincident aufgetreten. Unpatcheschene Schwachpunkte in unserer Microsoft Azure-Setup-Konfiguration wurden identifiziert. Obwohl Sicherheitsprotokolle aktualisiert und Audits durchgeführt wurden, bestehen weiterhin Bedenken bezüglich der Datensicherheit.</t>
+          <t>Können detaillierte Anleitungen zur Sicherung medizinischer Daten in Microsoft Teams unter Verwendung von Django 3.2 für Krankenhäuser bereitgestellt werden? Es ist entscheidend, dass die Sicherheit und Vertraulichkeit der Patientendaten gewährleistet sind. Bitte geben Sie Anleitungen zur Umsetzung von Sicherheitsmaßnahmen und zur Einhaltung der Vorschriften an.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1748</v>
+        <v>12618</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -507,20 +507,24 @@
           <t>Technischer Support</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Datenverlust-Ereignis in Gesundheitsversorgungssystem</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Wir möchten Sie darüber in Kenntnis setzen, dass eine potenzielle Datenexposition die IT-Systeme des Krankenhauses betrifft. Das Problem wurde bei einem Gesundheitsdienstleister festgestellt und scheint möglicherweise mit veralteten Sicherheitseinrichtungen im NAS-Netzwerk zusammenzuhängen. Erste Überprüfungen wurden mit aktualisierter McAfee-Software durchgeführt, und Verstöße wurden bestätigt. Wir nehmen diese Angelegenheit ernst und überwachen die Situation weiterhin. Weitere Updates werden bei Bedarf bereitgestellt.</t>
+          <t>Beim Gesundheitsversorgungssystem ist ein Datensicherheitsincident aufgetreten. Unpatcheschene Schwachpunkte in unserer Microsoft Azure-Setup-Konfiguration wurden identifiziert. Obwohl Sicherheitsprotokolle aktualisiert und Audits durchgeführt wurden, bestehen weiterhin Bedenken bezüglich der Datensicherheit.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>27831</v>
+        <v>1748</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kundenservice</t>
+          <t>Vertriebsanfrage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -528,24 +532,20 @@
           <t>Technischer Support</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>PyCharm Problem</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Ich habe Probleme mit PyCharm Professional 2021.1 unter Ubuntu. Das Systemupdates lädt korrekt, aber wenn ich versuche, die abhängigkeiten zu aktualisieren, besteht das Problem weiterhin.</t>
+          <t>Wir möchten Sie darüber in Kenntnis setzen, dass eine potenzielle Datenexposition die IT-Systeme des Krankenhauses betrifft. Das Problem wurde bei einem Gesundheitsdienstleister festgestellt und scheint möglicherweise mit veralteten Sicherheitseinrichtungen im NAS-Netzwerk zusammenzuhängen. Erste Überprüfungen wurden mit aktualisierter McAfee-Software durchgeführt, und Verstöße wurden bestätigt. Wir nehmen diese Angelegenheit ernst und überwachen die Situation weiterhin. Weitere Updates werden bei Bedarf bereitgestellt.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>16751</v>
+        <v>27831</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rechnung/Zahlung</t>
+          <t>Kundenservice</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -555,22 +555,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Datensperrern in Krankenhaus-IT-Systemen</t>
+          <t>PyCharm Problem</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Es wurde ein Datensperrern in den Krankenhaus-IT-Systemen festgestellt, der Patientenmedikationsdaten betreffen könnte. Dieser Sperrern könnte aufgrund veralteter Software-Vulnerabilitäten bei Python Produkten aufgetreten sein. Obwohl erste Sicherheitsprüfungen durchgeführt wurden, besteht das Problem weiterhin. Dringend benötigen wir Hilfe, um das Problem zu lösen und die Sicherheit der Patientendaten zu gewährleisten.</t>
+          <t>Ich habe Probleme mit PyCharm Professional 2021.1 unter Ubuntu. Das Systemupdates lädt korrekt, aber wenn ich versuche, die abhängigkeiten zu aktualisieren, besteht das Problem weiterhin.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>21969</v>
+        <v>16751</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Reklamation/Rückgabe</t>
+          <t>Rechnung/Zahlung</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -580,22 +580,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Sicherheitsverletzung in der Krankenhausauftragsysteme</t>
+          <t>Datensperrern in Krankenhaus-IT-Systemen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bitte Unterstützung einleiten</t>
+          <t>Es wurde ein Datensperrern in den Krankenhaus-IT-Systemen festgestellt, der Patientenmedikationsdaten betreffen könnte. Dieser Sperrern könnte aufgrund veralteter Software-Vulnerabilitäten bei Python Produkten aufgetreten sein. Obwohl erste Sicherheitsprüfungen durchgeführt wurden, besteht das Problem weiterhin. Dringend benötigen wir Hilfe, um das Problem zu lösen und die Sicherheit der Patientendaten zu gewährleisten.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>11541</v>
+        <v>21969</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Rechnung/Zahlung</t>
+          <t>Reklamation/Rückgabe</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -605,43 +605,47 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hilfe benötigt für Sicherheitsissue</t>
+          <t>Sicherheitsverletzung in der Krankenhausauftragsysteme</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Es wurde ein autorisierter Zugriff auf medizinische Daten gemeldet, der wahrscheinlich auf einen Mangel an Sicherheitsprotokollen zurückzuführen ist.</t>
+          <t>Bitte Unterstützung einleiten</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20301</v>
+        <v>11541</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Reklamation/Rückgabe</t>
+          <t>Rechnung/Zahlung</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vertriebsanfrage</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hilfe benötigt für Sicherheitsissue</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>geehrte Kundenservice-Team, kontaktiere Zusammenhang Datenanalyse-Dienstleistungen, Optimierung Investitionsstrategien anbieten. Könnten detaillierte Informationen angebotenen Dienstleistungen geben, einschließlich relevanter Fallstudien Empfehlungen? freuen, außerdem erklären könnten, Dienstleistungen beitragen, informierte Investitionsentscheidungen treffen. Bitte geben Auskunft Art Umfang Unterstützung, Kunden anbieten, zusätzliche Ressourcen gibt. Vielen Dank Zeit freue Rückmeldung bald.</t>
+          <t>Es wurde ein autorisierter Zugriff auf medizinische Daten gemeldet, der wahrscheinlich auf einen Mangel an Sicherheitsprotokollen zurückzuführen ist.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>6047</v>
+        <v>20301</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Kundenservice</t>
+          <t>Reklamation/Rückgabe</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -652,13 +656,13 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bitte teilen Sie uns die aktuellen Strategien im Bereich Digitalmarketing für Produkte mit. Wir möchten die neuesten Taktiken zur Steigerung des Marktwachstums und zur Optimierung der Technologieprodukte besprechen, um Ihre Anforderungen besser zu verstehen. Könnten Sie uns bitte zusätzliche Informationen zu den gegenwärtigen Strategien Ihrer Produkte zukommen lassen? Anschließend werden wir geeignete, aktualisierte Digitalmarketing-Strategien vorschlagen. Wir würden gerne einen Termin für einen Anruf vereinbaren, um weitere Details zu klären. Bitte teilen Sie uns mögliche Zeiten mit.</t>
+          <t>geehrte Kundenservice-Team, kontaktiere Zusammenhang Datenanalyse-Dienstleistungen, Optimierung Investitionsstrategien anbieten. Könnten detaillierte Informationen angebotenen Dienstleistungen geben, einschließlich relevanter Fallstudien Empfehlungen? freuen, außerdem erklären könnten, Dienstleistungen beitragen, informierte Investitionsentscheidungen treffen. Bitte geben Auskunft Art Umfang Unterstützung, Kunden anbieten, zusätzliche Ressourcen gibt. Vielen Dank Zeit freue Rückmeldung bald.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>6717</v>
+        <v>6047</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -673,7 +677,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Die digitale Kampagnen-Marketingagentur erreicht nicht die erwartete Markenentwicklung. Vermutlich liegt die Ursache im ineffektiven Targeting oder Messaging. Eine Überprüfung der Analysen und eine Anpassung der Anzeigenparameter wurden bereits unternommen.</t>
+          <t>Bitte teilen Sie uns die aktuellen Strategien im Bereich Digitalmarketing für Produkte mit. Wir möchten die neuesten Taktiken zur Steigerung des Marktwachstums und zur Optimierung der Technologieprodukte besprechen, um Ihre Anforderungen besser zu verstehen. Könnten Sie uns bitte zusätzliche Informationen zu den gegenwärtigen Strategien Ihrer Produkte zukommen lassen? Anschließend werden wir geeignete, aktualisierte Digitalmarketing-Strategien vorschlagen. Wir würden gerne einen Termin für einen Anruf vereinbaren, um weitere Details zu klären. Bitte teilen Sie uns mögliche Zeiten mit.</t>
         </is>
       </c>
     </row>
@@ -734,7 +738,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kundenservice</t>
+          <t>Technischer Support</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -759,7 +763,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Technischer Support</t>
+          <t>Kundenservice</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -953,7 +957,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>17533</v>
+        <v>16760</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -962,52 +966,52 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Technischer Support</t>
+          <t>Kundenservice</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Unterstützung für Rode NT-USB Mini</t>
+          <t>Veranschaulichung der Preise auf unserer Website - zusätzliche Erklärungen benötigt</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Können Sie Details zur Integration des Rode NT-USB Mini in Hospital-IT-Systeme zur Sicherung medizinischer Daten bereitstellen?</t>
+          <t>Ich schreibe Ihnen, um die Aktualisierung der Preisoptionen auf unserer Website zu veranlassen. Mehr Klärung soll das Verständnis der Kunden verbessern und ihnen dabei helfen, verständige Entscheidungen zu treffen. Missverständnisse sollen dadurch reduziert werden.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>22889</v>
+        <v>17533</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Reklamation/Rückgabe</t>
+          <t>Vertriebsanfrage</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Kundenservice</t>
+          <t>Technischer Support</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Anforderungen an erweiterte Sicherheitsprotokolle für medizinische Daten in Krankenhaus-IT-Systemen</t>
+          <t>Unterstützung für Rode NT-USB Mini</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Es wird vorgeschlagen, erweiterte Sicherheitsprotokolle für medizinische Daten in Krankenhaus-IT-Systemen umzusetzen, um die Sicherheit dieser Produkte zu gewährleisten.</t>
+          <t>Können Sie Details zur Integration des Rode NT-USB Mini in Hospital-IT-Systeme zur Sicherung medizinischer Daten bereitstellen?</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2837</v>
+        <v>22889</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Technischer Support</t>
+          <t>Reklamation/Rückgabe</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1017,47 +1021,47 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Anfrage zu Digitalen Strategien und Fördermöglichkeiten</t>
+          <t>Anforderungen an erweiterte Sicherheitsprotokolle für medizinische Daten in Krankenhaus-IT-Systemen</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Sehr geehrter Kundendienst, ich möchte mich erkundigen, wie die Förderung digitaler Strategien bei der Verwendung von AR-Brillen, Google Nest Wifi Routern usw. aussehen könnte. Könnten Sie bitte weitere Informationen und Ansätze bereitstellen, um die Bekanntheit zu erhöhen und den Verkauf der Produkte zu fördern? Besonders interessieren mich Details zu Marketingmaßnahmen, einschließlich Social-Media-Kampagnen, Influencer-Partnerschaften und Werbekanälen. Über eine Rückmeldung würde ich mich sehr freuen, um die Maßnahmen besser zu verstehen. Vielen Dank für Ihre Zeit. Ich freue mich auf Ihre Antwort.</t>
+          <t>Es wird vorgeschlagen, erweiterte Sicherheitsprotokolle für medizinische Daten in Krankenhaus-IT-Systemen umzusetzen, um die Sicherheit dieser Produkte zu gewährleisten.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>5046</v>
+        <v>2837</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Reklamation/Rückgabe</t>
+          <t>Technischer Support</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Technischer Support</t>
+          <t>Vertriebsanfrage</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Fehler beim fehlgeschlagenen Daten-Upload</t>
+          <t>Anfrage zu Digitalen Strategien und Fördermöglichkeiten</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Sehr geehrter Kundendienst, ich möchte ein Problem mit der Investment-Analytics-Plattform unseres Unternehmens melden. Kürzlich wurden Daten-Uploads auf der Plattform durchgeführt, jedoch trat ein Fehler auf, vermutlich infolge eines kürzlichen Software-Updates. Erste Versuche zur Fehlerbehebung umfassten einen Neustart des Systems und die Überprüfung der Integrität unserer Daten-Dateien, doch das Problem besteht weiterhin. Bei weiteren Versuchen, den Fehler einzugrenzen, wurden die Systemprotokolle überprüft und der Daten-Upload-Prozess kontrolliert, jedoch konnte die Ursache nicht ermittelt werden. Wir würden eine schnelle Unterstützung bei der Lösung des Problems sehr schätzen.</t>
+          <t>Sehr geehrter Kundendienst, ich möchte mich erkundigen, wie die Förderung digitaler Strategien bei der Verwendung von AR-Brillen, Google Nest Wifi Routern usw. aussehen könnte. Könnten Sie bitte weitere Informationen und Ansätze bereitstellen, um die Bekanntheit zu erhöhen und den Verkauf der Produkte zu fördern? Besonders interessieren mich Details zu Marketingmaßnahmen, einschließlich Social-Media-Kampagnen, Influencer-Partnerschaften und Werbekanälen. Über eine Rückmeldung würde ich mich sehr freuen, um die Maßnahmen besser zu verstehen. Vielen Dank für Ihre Zeit. Ich freue mich auf Ihre Antwort.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>15944</v>
+        <v>5046</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Rechnung/Zahlung</t>
+          <t>Reklamation/Rückgabe</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1067,22 +1071,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Verschlüsselung medizinischer Daten in PostgreSQL</t>
+          <t>Fehler beim fehlgeschlagenen Daten-Upload</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Sehr geehrte Kundensupport, wir schreiben im Anschluss unserer Anfrage zur Verschlüsselung medizinischer Daten in PostgreSQL-Systemen von Krankenhausauftritten. Wir suchen Rat zur Implementierung umfassender Sicherheitsmaßnahmen, um sensible Patientendaten zu schützen. Könnten Sie Empfehlungen zur Verschlüsselung, Zugriffskontrolle und Rettungsvorschriften geben? Wir freuen uns darauf, weitere Empfehlungen zu gängigen Praktiken zu erhalten. Vielen Dank für Ihre Zeit und Hilfe. Wir freuen uns darauf, bald von Ihnen zu hören.</t>
+          <t>Sehr geehrter Kundendienst, ich möchte ein Problem mit der Investment-Analytics-Plattform unseres Unternehmens melden. Kürzlich wurden Daten-Uploads auf der Plattform durchgeführt, jedoch trat ein Fehler auf, vermutlich infolge eines kürzlichen Software-Updates. Erste Versuche zur Fehlerbehebung umfassten einen Neustart des Systems und die Überprüfung der Integrität unserer Daten-Dateien, doch das Problem besteht weiterhin. Bei weiteren Versuchen, den Fehler einzugrenzen, wurden die Systemprotokolle überprüft und der Daten-Upload-Prozess kontrolliert, jedoch konnte die Ursache nicht ermittelt werden. Wir würden eine schnelle Unterstützung bei der Lösung des Problems sehr schätzen.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3051</v>
+        <v>15944</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Reklamation/Rückgabe</t>
+          <t>Rechnung/Zahlung</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1092,43 +1096,39 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Bericht über Synchronisierungsprobleme bei HelloSign auf Android 12 Geräten</t>
+          <t>Verschlüsselung medizinischer Daten in PostgreSQL</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sehr geehrter Kundendienst, Nutzer berichten von Synchronisierungsstörungen bei HelloSign auf Android 12 unter Debian 10 Buster. Verzögerungen bei der Aktualisierung von Unterschriftsdokumenten treten auf. Das Problem scheint auf Kompatibilitätsprobleme mit den neuesten Betriebssystemversionen von HelloSign zurückzuführen zu sein. Trotz Versuchen, die App neu zu installieren, die Netzwerkeinstellungen zurückzusetzen und die betroffene Software zu aktualisieren, sind keine Verbesserungen sichtbar. Die Synchronisationsprobleme beeinträchtigen weiterhin die Effizienz der Arbeitsabläufe. Wir bitten höflich um Ihre Unterstützung bei der schnellen Lösung des Problems, um weitere Verzögerungen zu vermeiden.</t>
+          <t>Sehr geehrte Kundensupport, wir schreiben im Anschluss unserer Anfrage zur Verschlüsselung medizinischer Daten in PostgreSQL-Systemen von Krankenhausauftritten. Wir suchen Rat zur Implementierung umfassender Sicherheitsmaßnahmen, um sensible Patientendaten zu schützen. Könnten Sie Empfehlungen zur Verschlüsselung, Zugriffskontrolle und Rettungsvorschriften geben? Wir freuen uns darauf, weitere Empfehlungen zu gängigen Praktiken zu erhalten. Vielen Dank für Ihre Zeit und Hilfe. Wir freuen uns darauf, bald von Ihnen zu hören.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>7342</v>
+        <v>2685</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Reklamation/Rückgabe</t>
+          <t>Rechnung/Zahlung</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Technischer Support</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Gefährdung der medizinischen Datensicherheit im Krankenhaus</t>
-        </is>
-      </c>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Die Sicherheit der medizinischen Daten im Krankenhaus wurde beeinträchtigt, möglicherweise durch veraltete Systemsoftware. Versuche, die Redis-Firewall-Einstellungen zu aktualisieren, führten zur Behebung des Problems. Trotz dieser Maßnahmen bestehen weiterhin Schwierigkeiten bei der Sicherung der medizinischen Daten.</t>
+          <t>Sehr geehrter Kundenservice, ich möchte mich nach Rechnungsdetails, Zahlungsoptionen, den angebotenen Dienstleistungen einer Marketingagentur sowie deren Beitrag zum Marktwachstum erkundigen. Könnten Sie bitte eine detaillierte Aufstellung der anfallenden Kosten sowie der akzeptierten Zahlungsmethoden bereitstellen? Ich würde auch gerne erfahren, ob es spezielle Rabatte oder Aktionen gibt. Zusätzlich interessiert mich, ob zusätzliche Gebühren anfallen, die ich beachten sollte. Ich bin daran interessiert, mehr über die angebotenen Dienstleistungen der Marketingagentur zu erfahren, um das Marktwachstum zu unterstützen. Vielen Dank im Voraus.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3132</v>
+        <v>3051</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1142,18 +1142,18 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Schwachstellen im Schutz medizinischer Daten</t>
+          <t>Bericht über Synchronisierungsprobleme bei HelloSign auf Android 12 Geräten</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Sehr geehrter Kundenservice, ich möchte auf Sicherheitslücken bei der Absicherung medizinischer Daten in Krankenhaus-IT-Systemen aufmerksam machen. Gesundheitsdienstleister könnten aufgrund unzureichender Verschlüsselung und veralteter Software auf Probleme stoßen. Erste Maßnahmen zur Behebung des Problems umfassten das Ändern von Passwörtern und die Anwendung grundlegender Software-Updates, jedoch wurde das Problem dadurch nicht vollständig gelöst. Ich bin besorgt über die möglichen Risiken im Zusammenhang mit diesen Schwachstellen, insbesondere hinsichtlich Datenverletzungen und unbefugtem Zugriff auf sensible medizinische Informationen. Ich bitte um eine dringende Prüfung dieser Angelegenheit und um eine umfassende Lösung.</t>
+          <t>Sehr geehrter Kundendienst, Nutzer berichten von Synchronisierungsstörungen bei HelloSign auf Android 12 unter Debian 10 Buster. Verzögerungen bei der Aktualisierung von Unterschriftsdokumenten treten auf. Das Problem scheint auf Kompatibilitätsprobleme mit den neuesten Betriebssystemversionen von HelloSign zurückzuführen zu sein. Trotz Versuchen, die App neu zu installieren, die Netzwerkeinstellungen zurückzusetzen und die betroffene Software zu aktualisieren, sind keine Verbesserungen sichtbar. Die Synchronisationsprobleme beeinträchtigen weiterhin die Effizienz der Arbeitsabläufe. Wir bitten höflich um Ihre Unterstützung bei der schnellen Lösung des Problems, um weitere Verzögerungen zu vermeiden.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>15516</v>
+        <v>7342</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1167,35 +1167,85 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Antrag auf hohe Priorität für Umstellung</t>
+          <t>Gefährdung der medizinischen Datensicherheit im Krankenhaus</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bitte Kompatibilität und Integrationsfunktionen betreffender Software- und Hardwareprodukte zu verbessern und das Gesamtleistungsniveau für das Benutzererlebnis zu optimieren.</t>
+          <t>Die Sicherheit der medizinischen Daten im Krankenhaus wurde beeinträchtigt, möglicherweise durch veraltete Systemsoftware. Versuche, die Redis-Firewall-Einstellungen zu aktualisieren, führten zur Behebung des Problems. Trotz dieser Maßnahmen bestehen weiterhin Schwierigkeiten bei der Sicherung der medizinischen Daten.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
+        <v>3132</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Schwachstellen im Schutz medizinischer Daten</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte auf Sicherheitslücken bei der Absicherung medizinischer Daten in Krankenhaus-IT-Systemen aufmerksam machen. Gesundheitsdienstleister könnten aufgrund unzureichender Verschlüsselung und veralteter Software auf Probleme stoßen. Erste Maßnahmen zur Behebung des Problems umfassten das Ändern von Passwörtern und die Anwendung grundlegender Software-Updates, jedoch wurde das Problem dadurch nicht vollständig gelöst. Ich bin besorgt über die möglichen Risiken im Zusammenhang mit diesen Schwachstellen, insbesondere hinsichtlich Datenverletzungen und unbefugtem Zugriff auf sensible medizinische Informationen. Ich bitte um eine dringende Prüfung dieser Angelegenheit und um eine umfassende Lösung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>15516</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Antrag auf hohe Priorität für Umstellung</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Bitte Kompatibilität und Integrationsfunktionen betreffender Software- und Hardwareprodukte zu verbessern und das Gesamtleistungsniveau für das Benutzererlebnis zu optimieren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
         <v>8809</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>Rechnung/Zahlung</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Vertriebsanfrage</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>Unterstützung für Datenanalyse</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Können detaillierte Dokumentationen, Anleitungen, Datenanalyselösungen und Optimierungsideen für Investitionen bereitstellen? Insbesondere helfen Verständnis für Werkzeuge, Portfolio-Management und Risikobewertung. Sind Fallstudien und Whitepapers verfügbar, um die Effektivität unserer Lösungen zu demonstrieren? Ich schätze die verfügbaren Informationen und kann die Angebote besser verstehen, um meine Investitionsstrategie zu fördern. Vielen Dank für Ihre Unterstützung.</t>
         </is>

</xml_diff>

<commit_message>
LLM-Lauf auf 300 Testtickets, Baseline speichert Vorhersagen und Zeiten, Spalte Wahr in Label umbenannt, Lizenz ergänzt
</commit_message>
<xml_diff>
--- a/results/fehleranalyse.xlsx
+++ b/results/fehleranalyse.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1203,7 +1203,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>15516</v>
+        <v>8970</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1212,42 +1212,4043 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Technischer Support</t>
+          <t>Kundenservice</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Antrag auf hohe Priorität für Umstellung</t>
+          <t>Auswirkungen der Marketingstrategie auf Produktretouren</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bitte Kompatibilität und Integrationsfunktionen betreffender Software- und Hardwareprodukte zu verbessern und das Gesamtleistungsniveau für das Benutzererlebnis zu optimieren.</t>
+          <t>Sehr geehrter Kundenservice, ich schreibe, um auf ein Problem aufmerksam zu machen, das die Marketingagentur betrifft. Es kommt häufig zu Produktretouren und Umtauschaktionen, was das Markenwachstum negativ beeinflusst. Trotz unserer Bemühungen, die Zielgruppensegmentierung zu verfeinern und die Produktbeschreibungen zu verbessern, wurden keine signifikanten Verbesserungen bei den Rücklaufquoten festgestellt. Es ist möglich, dass die digitale Zielgruppenansprache falsche Kundenerwartungen weckt. Wir würden eine Unterstützung oder Anleitung begrüßen, um dieses Problem anzugehen und die allgemeine Kundenzufriedenheit zu steigern. Vielen Dank für Ihre Zeit und Unterstützung. Mit freundlichen Grüßen,</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
+        <v>15516</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Antrag auf hohe Priorität für Umstellung</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Bitte Kompatibilität und Integrationsfunktionen betreffender Software- und Hardwareprodukte zu verbessern und das Gesamtleistungsniveau für das Benutzererlebnis zu optimieren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
         <v>8809</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Rechnung/Zahlung</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Vertriebsanfrage</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>Unterstützung für Datenanalyse</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Können detaillierte Dokumentationen, Anleitungen, Datenanalyselösungen und Optimierungsideen für Investitionen bereitstellen? Insbesondere helfen Verständnis für Werkzeuge, Portfolio-Management und Risikobewertung. Sind Fallstudien und Whitepapers verfügbar, um die Effektivität unserer Lösungen zu demonstrieren? Ich schätze die verfügbaren Informationen und kann die Angebote besser verstehen, um meine Investitionsstrategie zu fördern. Vielen Dank für Ihre Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>22311</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Unterstützung für digitale Marketingstrategien erforderlich</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Mehr Details zu Strategien benötigt?</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>13764</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Es gibt Bedenken bezüglich unerlaubter Zugriff Versuche auf medizinische Daten. Schwache Firewall-Konfiguration könnte die Ursache sein. Zugriffssteuerungen wurden verfestigt und Sicherheitsprotokolle aktualisiert, dennoch bestehen Anliegen hinsichtlich fortbestehender Schwachstellen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>24546</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, ich schreibe, um Näheres über Rechnungsstellungsrichtlinien für Puppet- Smartwatch-Integrationen und SaaS-Plattform zu erfahren. Bitte geben Sie detaillierte Informationen und berechnen Sie die Integrationen. Zudem würde ich relevante Dokumentationen und Ressourcen zu sehen bekommen schätzen. Darüber hinaus möchte ich wissen, welche speziellen Anforderungen und speziellen Setup-Prozesse für die Integrationen erforderlich sind. Danke für Ihre Unterstützung und freue mich auf Ihre Rückmeldung. freundliche Grüße, [Ihr Name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>25079</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Daten Disparaten</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Es wurden unerwartete Daten Disparaten erkannt, während Analysen, Rückzahlungen und Austausche durchgeführt wurden. Diese Disparaten scheinen aufgrund einer neueren Software-aktualisierung aufgetreten zu sein. Die betroffenen Datensätze wurden bereits manuell überprüft und es wurde versucht, die Analysewerkzeuge neu zu kalibrieren, jedoch ohne Erfolg. Bitte helfen Sie bei der Lösung dieses Problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>24757</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Informationsmaterial zu Datensicherheitslösungen für Gesundheitsorganisationen</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Könnten Sie detaillierte Informationen zu Datensicherheitslösungen für Gesundheitsorganisationen geben? Wir möchten mehr darüber erfahren, wie wir sensible Patientendaten vor Einblicken schützen können, die Vorschriften erschweren. Vielen Dank für Ihre Unterstützung. Wir freuen uns darauf, bald von Ihnen zu hören.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>18524</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Anfrage zu Sicherheitsfall</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Lieber Kundenservice, wir möchten auf einen Sicherheitsfall hinweisen, bei dem unautorisiertes Zugriff auf medizinische Datensysteme erfolgte. Dieser Vorgang ist auf Verstoß gegen veraltete Sicherheitsprotokolle zurückzuführen. Bitte beheben Sie den Fall, aktualisieren Sie die Software, überprüfen Sie Zugriffslöcher und stärken Sie die Passwortsicherheitsrichtlinien. Wir schätzen Ihre Bemühungen zur Sicherstellung der Integrität unserer Systeme und empfehlen Ihnen, eine umfassende Risikobewertung und einen Vernetzungsscan durchzuführen, um mögliche Schwachstellen zu identifizieren. Bitte geben Sie uns Anweisungen zu Ihren nächsten Schritten. Vielen Dank für Ihre Unterstützung bei dieser Angelegenheit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>7889</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Integrationsproblem bei mehreren Diensten</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Fehler beim Abgleichen von Slack mit QuickBooks Online</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>19185</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Probleme mit Software-Updates: Kompatibilität Microsoft OneNote, Malwarebytes 4.4</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Neueste Updates verursachen Probleme mit Microsoft OneNote und Malwarebytes 4.4, was Aufgaben stört. Rollback- und Neinstallationsversuche waren unerfolgreich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>5028</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Digitale Marketingansätze für Markenentwicklung</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Könnten Sie bitte die spezifischen digitalen Taktiken mitteilen, die die Marketingagentur nutzt, um das Wachstum der Marke effizient zu fördern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>7863</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Erweiterte Sicherheitsmaßnahmen für Daten im Gesundheitswesen</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich über die Implementierung erweiterter Sicherheitsprotokolle für Krankenhaus-IT-Systeme und Plattformen zur Verwaltung medizinischer Daten erkundigen. Dieses wichtige Thema erfordert sofortige Aufmerksamkeit, um die Vertraulichkeit, Integrität und Verfügbarkeit sensibler Patientendaten sicherzustellen. Ich bitte um zusätzliche Informationen zu bewährten Verfahren und verfügbaren Lösungen, um diese Angelegenheit anzugehen. Bitte stellen Sie detaillierte Anweisungen bereit, damit wir die Initiative entsprechend umsetzen können. Ich freue mich auf eine schnelle Rückmeldung und darauf, bald von Ihnen zu hören. Vielen Dank für Ihre Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>25024</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Betonen Sie die Erhöhung der Datensicherheitsprotokolle</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Die Schutzmaßnahmen für die IT-Infrastruktur des Krankenhauses, insbesondere für medizinische Akten, sollten verbessert werden. Dieser Prozess umfasst die Erweiterung der bestehenden Datensicherheitsrichtlinien, einschließlich der Implementierung robusterer Firewalls, der Verschlüsselung sensibler Daten, regelmäßiger Sicherheitsaktualisierungen und der Ausbildung des Personals. Ziel ist es, die Vertraulichkeit und Unversehrtheit der Patientendaten zu gewährleisten und so das Vertrauen in die Gesundheitsdienstleistungen zu erhalten. Der Einhalt der gesetzlichen Anforderungen ist notwendig, um qualitativ hochwertige Pflege zu bieten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>26004</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Digitaler Markenentwicklungswachstum</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Wir fordern Änderungen an Ihren Strategien, um das Markenwachstum der betroffenen Produkte durch effizientere Marketingkampagnen zu fördern und die Verkaufszahlen sowie den Umsatz zu verbessern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>23455</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Details zur Tarifkarte für Kubernetes-Integration</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Könnten Sie mir die genauen Details der Tarife für die Kubernetes-Integration liefern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>26307</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Sicherheitsprobleme im Gesundheitsdienstleistungsbereich</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Es gab einen Datenverlust, bei dem die medizinischen Akten auf dem IT-System des Krankenhauses beschädigt wurden. Wahrscheinlich sind veraltete Sicherheitsprotokolle die Ursache, die Mitarbeiterinnen und Mitarbeiter durch Phishingversuche betrogen wurden. Momentan sind Zugriffsbeschränkungen in Kraft und eine detaillierte Sicherheitsprüfung wurde gestartet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>25351</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Detaillierte Anleitungen zur PyTorch-Datenanalyse</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Können detaillierte Anleitungen zur effektiven Nutzung von PyTorch für Datenanalyse und Optimierung von Investitionen bereitstellen? Dies soll helfen, informierte Entscheidungen zu treffen und maximalen Ertrag zu erzielen. Vielen Dank für Ihre Zeit und Hilfe bei dieser Angelegenheit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>27186</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Bündeln zusätzlicher Tools zur Steigerung der Projektmanagement Effizienz</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Gehrte Kundenservice, ich schreibe an, um die Integration zusätzlicher Drittanbieter-Tools für Projektmanagement-Software-as-a-Service (SaaS) zu fordern. Ich wäre dankbar für Unterstützung bei der Integration von Babbel, Google Translate und Adobe Premiere Pro. Diese Tools könnten den Arbeitsablauf und die Produktivität erheblich verbessern. Die Integration von Babbel würde den Sprachkenntnissen der Teammitglieder helfen, Google Translate würde die Kommunikation mit internationalen Kunden erleichtern, und Adobe Premiere Pro würde es ermöglichen, hochwertige Videokonten zu erstellen. Ich glaube, die Integration dieser Tools könnte einen großen Mehrwert gegenüber Konkurrenten bieten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>18058</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Ich interessiere mich für digitale Markenstrategien und würde gerne mehr darüber erfahren. Könnten Sie mir Methoden zur Förderung des Markenwachstums nennen? Ich möchte verstehen, wie Techniken eingesetzt werden können, um die Markenpräsenz und den Engagezustand zu erhöhen. Ihre Expertise schätze ich sehr. Vielen Dank!</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>12246</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Optimierung digitaler Strategien Crucial MX500 1TB SSD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, ich möchte um Informationen zur Optimierung digitaler Strategien für den Crucial MX500 1TB SSD bitten. Könnten Sie detaillierte Einblicke in Maßnahmen geben, die die Leistung und Lebensdauer des SSDs verbessern? Ich freue mich auf Empfehlungen zu Tipp und Tricks, die mir helfen können. Darüber hinaus interessiert mich, ob es spezifische Softwarewerkzeuge gibt, die die Optimierung von SSDs unterstützen. Bitte geben Sie mir an, welche weiteren Informationen Sie benötigen. Vielen Dank für Ihre Unterstützung und die Zeit, die Sie mir gewähren. Ich freue mich darauf zu hören.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>24846</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Kontaktieren Sie uns, um Informationen über die Verwendung von medizinischen Daten im Netgear Nighthawk Mesh Wi-Fi 6 System zu erhalten. Möchten Sie Details zum Verfahren, wie die Gewährleistung der Vertraulichkeit und Integrität sensibler medizinischer Informationen über das Netzwerk übertragen werden, erfahren? Wir freuen uns, Anleitungen zur Konfiguration zusätzlicher Sicherheitsmaßnahmen zu geben, um die Daten zu schützen. Empfehlen wir, WPA3-Verschlüsselung zu aktivieren und nicht-medizinische Geräte in ein Gastschaltungsnetzwerk zu integrieren. Darüber hinaus sollten Sie in Betracht ziehen, einen virtuellen privaten Netzwerk (VPN) zu konfigurieren, um sicherzustellen, dass die Datenübertragungen sicher sind. Gibt es die Möglichkeit, über die Konfiguration von Netzwerksegmentierung zu sprechen, um den medizinischen Datenerverkehr abzuschirmen? Wir sind bereit, spezifische Anleitungen zur Konfiguration telefonisch zu besprechen. Ein Anruf zur Diskussion der Detailkonfigurationen wäre angemessen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>8804</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte um eine Aktualisierung der Produktintegration bezüglich der Kompatibilität der aufgeführten Software- und Hardware-Komponenten bitten. Die derzeitige veraltete Integration verursacht Schwierigkeiten im Arbeitsablauf. Daher bitte ich darum, die Integration auf die neueste Version zu aktualisieren, um eine reibungslose Kompatibilität zu gewährleisten. Ein Update würde dem Team ermöglichen, effizienter und effektiver zu arbeiten. Wir würden eine schnelle Lösung sehr schätzen. Vielen Dank für Ihre Zeit und Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>5945</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Sicherheitsproblem: Verletzung von Gesundheitsdaten</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundendienst, hiermit möchte ich ein kritisches Sicherheitsproblem im Zusammenhang mit der Datensicherheit eines Gesundheitsdienstleisters melden. Kürzlich kam es zu einer Datenpanne, bei der medizinische Informationen gefährdet wurden. Die Verletzung wurde vermutlich durch veraltete Cassandra- und NAS-Systeme ausgenutzt, die bekannte Schwachstellen aufweisen. Wir haben versucht, das Problem durch erste Scans sowie durch das Einspielen von Patch-Updates für Cassandra und das NAS-System mithilfe von JIRA Software zu beheben. Bedauerlicherweise besteht das Problem weiterhin. Ich bitte um schnelle Unterstützung bei der Lösung dieses Problems und um Informationen zu den nächsten Schritten. Ich schätze Ihre zügige Aufmerksamkeit für dieses Anliegen. Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>26828</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Sicherheitslücke in KI-Systemen des Krankenhauses</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Obwohl die Antivirussoftware aktualisiert wurde, bestehen immer noch Schwachstellen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>28376</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Ausführen der Aktualisierung der Marketingstrategien</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Lieber Kundenservice, ich möchte die Aktualisierung unserer digitalen Marketingstrategien beantragen, um die Markenpräsenz und die Engagementschaffung auf verschiedenen Plattformen sowie die Verbesserung der Produktpresenz zu verbessern. Da die aktuellen Strategien leider nicht den gewünschten Erfolg bringen, müssen wir unsere Ansätze überdenken, um im Wettbewerb erfolgreich zu bleiben. Ich schätze es, dass Sie Ratschläge zur Verbesserung unserer Marketingbemühungen geben könnten. Insbesondere interessiere ich mich für mehr Sozialmedienmarketing, Inhaltsmarketing und Suchmaschinenoptimierung. Ich glaube, dass eine Aktualisierung unserer Marketingstrategien dazu beitragen kann, unser Markenwissen zu erweitern und den Verkehr auf unserer Website zu erhöhen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>17695</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Probleme mit dem Datenauswertungsfernzeug</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Das Datenauswertungsfernzeug zeigt Leistungsschwierigkeiten, und der Datenabruf wird beeinträchtigt, möglicherweise aufgrund von Systemüberlastung oder Software-Configurationsfehler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>27270</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Sicherheitssystem Krankenhaus IT-System</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Es wurde ein Versuch unbefugten Zugriffs auf das Krankenhaus IT-System festgestellt. Dies beinhaltet ein Potenzial, das die Sicherheit medizinischer Daten der Patienten gefährdet. Maßnahmen, die untergenommen werden sollen, umfassen das Aktualisieren der Antiviren-Definitionen, das Prüfen der Zugriffsnachweise, um den Ursprung der Sicherheitslücke zu identifizieren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>10192</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Probleme mit der Integration von OBS Studio</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Es gibt Fehler nach der Integration von OBS Studio in ClickUp. Die Projektmanagement-Funktion wird aufgrund von Kompatibilitätsproblemen beeinträchtigt. Das Programm wurde neu gestartet und Updates wurden überprüft, aber das Problem behält sich bestehen. Es wird Unterstützung benötigt, um das Problem zu lösen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>26125</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Details zur Sicherung medizinischer Daten im IBM Cloud-Dienst</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Ich würde gerne mehr Informationen zu Sicherheitsfunktionen, Zertifizierungen, Speicherung und Verarbeitung medizinischer Daten im IBM Cloud-Dienst erhalten. Könnten Sie Details zu den verfügbaren IT-Dienstleistungen zur Sicherung medizinischer Daten liefern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>3160</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Enhanced Security for Medical Systems</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte anfragen, ob die Implementierung verbesserter Sicherheitsprotokolle und Updates für bestimmte Softwaregeräte erfolgen kann, um medizinische Daten in den IT-Systemen des Krankenhauses zu schützen. Es ist entscheidend, potenzielle Cyber-Bedrohungen zu verhindern und die Vertraulichkeit, Integrität sowie Verfügbarkeit sensibler Patientendaten sicherzustellen. Ich würde mich über weitere Informationen zu den bereits ergriffenen Maßnahmen sowie Vorschläge zur Behebung des Problems freuen. Bitte informieren Sie mich, wenn zusätzliche Maßnahmen ergriffen werden können, um die Sicherheit zu erhöhen. Ich freue mich auf eine zeitnahe Rückmeldung. Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>5421</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Rechnungsfehler-Meldung</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Unsere Agentur erlebt wiederkehrende Abrechnungsprobleme, die mehrere Produkte betreffen. Dies könnte auf Integrationsfehler zwischen Zahlungs-Gateways und der Produktdatenbank zurückzuführen sein. Wir haben Maßnahmen ergriffen, darunter die Neuverarbeitung von Rechnungen, Überprüfung der Zahlungssystemeinstellungen und Behebung von Diskrepanzen. Das Problem besteht weiterhin, und wir benötigen Unterstützung, um es so schnell wie möglich zu lösen und weitere Komplikationen zu vermeiden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>28558</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Unpräzise Berichte zur Verarbeitung von Investment-Daten</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Es gibt Unpräzisionen in den Berichten zur Verarbeitung von Investment-Daten. Mögliche Ursachen könnten veraltete Algorithmen sein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>2610</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Update der Digitalstrategie zur Steigerung des Markenwachstums</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte eine Aktualisierung unserer Integrationstools für die digitale Strategie anfragen. Das derzeitige Setup erfüllt unsere Bedürfnisse, doch wir streben eine Verbesserung des Markenwachstums und der Marketingeffizienz an. Wir sind überzeugt, dass die Integration der richtigen Tools unsere Online-Präsenz stärken, das Engagement erhöhen und den Umsatz steigern kann. Besonders interessiert sind wir an Updates für Social-Media-Management-Tools, E-Mail-Marketing-Software und Datenanalyseplattformen. Wir würden eine Empfehlung oder Anleitung schätzen, um die besten Tools und Integrationen für unser Unternehmen zu identifizieren. Außerdem möchten wir ein Treffen vereinbaren, um die digitalen Maßnahmen weiter zu besprechen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>19258</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Einfluss von Änderungen am Algorithmus auf die Kundenbindung gemessen durch Leistungsindikatoren</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Sehr geehrte [Name], wir entschuldigen uns für den Rückgang der Leistungsindikatoren in Bezug auf die Kundenbindung, der sich aufgrund von Änderungen im Algorithmus ergab. Wir möchten gerne dieses Thema genauer besprechen, um mögliche Lösungen zu verstehen. Bitte teilen Sie uns Ihre Beobachtungen mit, die die vorher erwarteten Indikatoren beeinflusst haben. Um das Problem zu prüfen, können wir telefonisch eine Besprechung vereinbaren unter [Telefonnummer], um mögliche Anpassungen zu besprechen und den Rückgang der Kundenbindung zu verbessern und zu reduzieren. Geben Sie uns bitte an, wann eine geeignete Zeit für die Besprechung verfügbar ist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>16991</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Bewerbung für Verbesserungen der Sicherheitsmaßnahmen</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Gehörte Kundenservice, schreibe Sie über die notwendigen Verbesserungen an den Sicherheitsmaßnahmen, insbesondere bei der Verwaltung medizinischer Daten und der IT-Infrastruktur von Krankenhäusern. Die Gewährleistung der Einhaltung der Datensicherheitsstandards ist entscheidender Bedeutung für die Gesundheitsbranche. Ich möchte vorschlagen, fortschrittliche Verschlüsselungsverfahren einzuführen, regelmäßige Sicherheitsprüfungen durchzuführen und Schulungen zum Umgang mit den besten Praktiken der Datenschutzverwaltung durchzuführen. Darüber hinaus wäre die Einrichtung eines Incidentschadensplans und die Durchführung regelmäßiger Penetrationstests, um Schwachstellen zu identifizieren, ein Vorteil. Ich glaube, dass diese Maßnahmen unsere medizinischen Daten und IT-Infrastruktur erheblich verbessern könnten. Ich freue mich auf eine Diskussion dieser Vorschläge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>7345</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich bin daran interessiert, mehr über Investitionsoptimierungsdienste zu erfahren und wie Datenanalysen dabei helfen können. Könnten Sie mir bitte detaillierte Informationen zu den Rechnungs- und Zahlungsoptionen Ihrer Dienste mitteilen? Ich möchte wissen, welche Zahlungsmethoden akzeptiert werden, ob es Rabatte für langfristige Verpflichtungen gibt und ob zusätzliche Gebühren für die Nutzung der Dienste anfallen. Ich freue mich darauf, mehr zu erfahren, wie Ihre Dienstleistungen bei der Optimierung meiner Investitionen unterstützen können. Vielen Dank für Ihre Zeit und Unterstützung. Mit freundlichen Grüßen, [Ihr Name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>5764</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Problem with Norton Integration</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich bitte um Unterstützung bei der Integration von Norton 360 Symantec Endpoint Protection 14.3 auf der SaaS-Plattform. Könnten Sie bitte eine Schritt-für-Schritt-Anleitung und Dokumentationen bereitstellen, die die erforderlichen Schritte für die Durchführung der Integration beschreiben? Zusätzliche Ressourcen oder Informationen, die eine erfolgreiche Integration gewährleisten, wären ebenfalls sehr willkommen. Vielen Dank im Voraus für Ihre Zeit und Unterstützung bei diesem Anliegen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>27466</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Probleme bei der Integration von Projektmanagement-Software mit drittanbieterdiensten</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Wir haben Schwierigkeiten bei der Integration unserer Projektmanagement-Software mit drittanbieterdiensten. Diese Probleme scheinen mit den neuesten API-Aktualisierungen zu zusammenhängen. Bislang haben wir die Updates rückgängig gemacht und den Cache geleert, aber das Problem behält sich bestanden. Ich schätze, es wäre hilfreich, wenn Sie uns helfen könnten, die Angelegenheit zu lösen, da die Produktivität dadurch beeinträchtigt wird. Bitte lassen Sie uns wissen, welche weiteren Schritte wir unternehmen können, falls Sie weitere Informationen benötigen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>2181</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Probleme bei der Daten-Synchronisierung in Finanzunternehmen auftreten</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundendienst, ich möchte ein dringendes Problem melden, das die Anlageanalysen betrifft. Das Finanzunternehmen hat Schwierigkeiten mit der Daten-Synchronisierung über mehrere Produkte hinweg, was die Fähigkeit erheblich beeinträchtigt, präzise Anlageinformationen bereitzustellen. Trotz wiederholter Versuche, die Systeme neu zu starten und die Datenquellen zu überprüfen, besteht das Problem weiterhin. Es wird vermutet, dass Konflikte bei der Integration die Ursache sein könnten. Wir würden eine schnelle Lösung des Problems sehr schätzen und wären dankbar für Ihre Unterstützung. Bitte informieren Sie uns, falls weitere Maßnahmen notwendig sind, die wir ergreifen können.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>13642</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Hilfe bei Social Media-Kampagne</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Die kürzlich gestartete Kampagne zeigte einen schlechteren Engagementquote als erwartet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>26788</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Support für Data Analytics</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Brauche zusätzliche Informationen über die Daten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>24327</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Optionen für die Integration von TensorFlow in das SaaS-Projekt</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Ich möchte mehr über die Integration von TensorFlow in eine SaaS-Projektmanagement-Lösung erfahren. Könnten Sie mir zusätzliche Informationen zu diesem Thema bereitstellen? Es wäre hilfreich, wenn Sie den Integrationsprozess, die Vorteile sowie eventuelle Herausforderungen beschreiben könnten. Vielen Dank für Ihre Unterstützung bei diesem Thema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>19061</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Könnten Sie mehr Details zum Thema digitale Strategien, Förderung und Markenentwicklung geben? Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>18488</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Unterstützung für FL Studio</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Ich würde gerne mehr Informationen zu den Supportoptionen von FL Studio 20.8 erhalten. Ich bin interessiert daran, mehr über die verfügbaren Ressourcen zu erfahren, um so das Softwarepaket am besten nutzen zu können. Vielen Dank für Ihre Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>2466</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Digitale Kampagnen sind erfolgreich</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte auf ein Problem aufmerksam machen, das meine Marketingaktivitäten beeinträchtigt. Die digitalen Kampagnen verzeichnen eine deutliche Abnahme der Interaktionen. Nach Recherchen vermuten wir, dass die Ursache möglicherweise in Softwareintegrationskonflikten zwischen mehreren Plattformen liegt. Wir haben versucht, die betroffenen Produkte zu aktualisieren und neu zu starten, jedoch blieb das Problem bestehen. Wir befürchten, dass unsere Fähigkeit, die Zielgruppe zu erreichen und unsere Marketingziele zu erfüllen, beeinträchtigt sein könnte. Könnten Sie bitte das Problem untersuchen und eine Anleitung zur Lösung bereitstellen?\"</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>19426</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Investment-Reporting-Issue Diagnose</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Begegnen Verzögerungen bei der Investment-Reporting-Funktion aufgrund von Problemen mit der Datensammlung, möglicherweise verursacht durch neueste Software-Updates. Trotz Versuche, die Datensysteme neu zu synchronisieren und Systeme neu zu starten, besteht das Problem weiterhin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>27823</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Verbesserung der Investitionsanalyseunterstützung mit IBM SPSS Statistics 28</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, bitten Sie, nachzufragen, welche Möglichkeiten IBM SPSS Statistics 28 bietet, um Investitionsanalyse und Datenanalysebereiche zu verbessern. Könnten Sie mehr Informationen zu den Möglichkeiten geben, wie das Softwarepaket Investitionsentscheidungen verbessern kann? Insbesondere interessiere ich mich für fortgeschrittene statistische Techniken, Datenvisualisierungstools und prognostische Modellierungsfähigkeiten. Unterstützt IBM SPSS Statistics 28 die Analyse großer Datensätze und die Identifikation von Trends und Mustern? Gibt es case studies oder Beispiele, die den Einsatz des Softwarepakets für Investitionsanalyse verdeutlichen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>4749</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Unstimmigkeiten in der Investitionsdatenanalyse</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Unregelmäßigkeiten in den Daten beeinträchtigen die Präzision bei der Entscheidungsfindung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>28038</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Anfrage zur Unterstützung von Pro Tools</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Ich schreibe, um nachzufragen, ob die Pro Tools SaaS-Project-Management-Lösung integriert werden kann. Bitte geben Sie mehr Informationen zum Thema. Ich freue mich, Ressourcen und Unterstützung anbieten zu können, um den Integrationsvorgang zu unterstützen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>5882</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Fehler bei der Abrechnungssoftware</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte einen Fehler in der Abrechnungssoftware melden, der bei Gesundheitsdienstleistern aufgetreten ist. Es scheint, dass mehrere Softwaregeräte betroffen sind, wobei vermutet wird, dass Systemintegrationsfehler die Ursache sein könnten. Das Team hat bereits versucht, die Dienste neu zu starten und die Kontodaten zu überprüfen, doch die Probleme bestehen weiterhin. Wir befürchten, dass diese Fehler finanzielle Verluste verursachen und die Abläufe stören könnten. Ich bitte um Unterstützung bei einer schnellen Lösung des Problems. Könnten Sie bitte das Problem untersuchen und eine Anleitung zur Behebung bereitstellen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>24748</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Frage zur sicheren Speicherung medizinischer Daten in Krankenhaus-IT-Systemen</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Könnten Sie bitte detaillierte Informationen über die Dienstleistungen zur Sicherung medizinischer Daten in Krankenhaus-IT-Systemen bereitstellen? Vielen Dank für Ihre Zeit und Hilfe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>28375</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Unterstützung für Investitionen</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Wir haben unerwartete Schwankungen in den Investitionsleistungen festgestellt, obwohl wir Datenanalysebemühungen unternommen haben. Die Probleme könnten auf ungenaue Datenintegration und Softwarekompabilitätsprobleme zurückzuführen sein. Wir haben verschiedene Dateneingaben überarbeitet und verschiedene Analysewerkzeuge getestet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>12962</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Probleme mit der Anmeldung nach der neuesten Aktualisierung</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice-Team, ich begehe aktive Anmeldefehler nach der Anwendung der neuesten Authentifizierungsserver-Aktualisierung. Ich habe versucht, den Browser-Cache zu leeren und das Passwort zu resetten, aber das Problem behält sich fort. Die Anmeldefehler sind sporadisch aufgetreten und machen es schwierig, eine Mustererkennung durchzuführen. Ich schätze Ihre Hilfe beim Auflösen dieses Problems in kürzester Zeit, um Benutzerstörungen zu minimieren. Bitte geben Sie mir weitere Schritte an, die ich ausführen kann, um das bekannte Problem zu lösen. Vielen Dank für Ihre schnelle Beachtung dieser Angelegenheit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>6797</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Unterstützung bei digitalen Werkzeugen</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Die Marketingagentur verzeichnet einen Leistungsabfall bei mehreren digitalen Tools, möglicherweise verursacht durch Integrationsprobleme. Erste Maßnahmen zur Fehlerbehebung umfassten Neustart der Geräte und das Löschen des Caches; das Problem besteht jedoch weiterhin. Wir benötigen schnelle Unterstützung, um das Problem zu beheben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>586</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Guidance for Incorporating Python-Based Models</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Sehr geehrtes Support-Team,
+ich hoffe, diese Nachricht erreicht Sie wohlbehalten. Momentan bin ich an einem Projekt beteiligt, das die Einbindung von auf Python beruhenden Machine-Learning-Modellen in bestehende Big-Data-See automatisierte Rebalancing-Algorithmen umfasst. Ziel ist es, Echtzeit-Analysen zu verbessern, um Anlageentscheidungen effizienter zu gestalten und die Leistungsfähigkeit der Strategien zu steigern.
+Aufgrund der Komplexität dieses Vorhabens suche ich Rat zu bewährten Verfahren, empfehlenswerten Tools sowie Plattformen und Frameworks, die eine nahtlose Verbindung zwischen Python-ML-Modellen und groß angelegten Datenspeicherungssystemen ermöglichen. Besonders interessiert bin ich daran zu verstehen,</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>8145</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Optimierung der Datenanalyse-Tools</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundendienst, ich möchte eine Anfrage zur Verbesserung der bei unserer Finanzfirma eingesetzten Datenanalyse-Tools stellen. Die aktuellen Funktionen sind eingeschränkt und erschweren das Erkennen von Echtzeit-Einblicken, was die Optimierung unserer Investitionen erschwert. Ich bin der Ansicht, dass eine erweiterte Datenanalyse fundierte Entscheidungen ermöglicht und die Renditen steigern kann. Daher bitte ich das Entwicklungsteam, die Integration prädiktiver Modellierungsfunktionen sowie maschineller Lernalgorithmen in die bestehenden Tools zu prüfen. Dies würde eine bessere Analyse von Markttrends und datenbasierte Entscheidungen erleichtern. Wir schätzen Ihre Prüfung unseres Anliegens und Ihre Einschätzung.
+Mit freundlichen Grüßen,
+[Name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>19245</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, wir haben Schwierigkeiten bei den Datenanalyseprozessen im SAP ERP-System. Das System brach beim Zusammenfassen der Analyse von Investitionsportfolios zusammen, möglicherweise aufgrund von Datenübertreibung oder Fehlkonfiguration. Versuche, um Abfragen zu optimieren und unnötige Daten zu löschen, blieben erfolglos. Wir benötigen Unterstützung, um das Problem zu lösen und zukünftige Systembrüche zu vermeiden. Bitte helfen Sie uns, die Ursache-Effekt-Verhältnisse zu identifizieren und eine Lösung anzubieten, um den Datenanalyseprozessen den gewünschten Fluss zu geben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>9616</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Integrationsschwierigkeiten bei Finanzdienstleister</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Finanzinstitut, Investitionsdatenanalyse verbessert, Schwierigkeiten bei der Integration mehrerer Produkte. Möglicherweise verursacht durch nicht kompatible Softwareversionen. Es wurden grundlegende Fehlerbehebungen und Software-Updates versucht, jedoch ohne Erfolg. Wir benötigen Unterstützung bei der Lösung des Problems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>13431</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Gehörte Kundenservice, ich schreibe Ihnen, um Fehler im Projektleitungssystem zu melden. Es tritt abwechselnd auf Gipfelzeiten Ausfälle auf, die möglicherweise auf Überlastung des Servers oder Netzwerkproblemen zurückzuführen sind. Trotz unserer Bemühungen, den Server zu optimieren und die Ressourcen zu erhöhen, beharrt das Problem weiterhin. Ich schätze Ihr Eingreifen, um die Lösung in der kürzesten Zeit zu untersuchen und anzubieten. Bitte informieren Sie mich, falls zusätzliche Informationen erforderlich sind, um die Untersuchung voranzutreiben. Ich stehe Ihnen gerne zur Verfügung, um notwendige Details zu besprechen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>10270</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Verbesserung des Markenwachstums durch digitale Strategien online</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, ich wende mich an Sie, um mehr über Methoden zur Erhöhung des Markenwachstums durch digitale Strategien zu erfahren. Könnten Sie mehr Informationen zu den Verfahren geben, die für die Erhöhung der Markenbewusstheit verwendet werden? Ich bin sehr daran interessiert, mehr Ansätze zu erfahren, die ich meinem Unternehmen anwenden kann. Ich freue mich auf Ihre Rückmeldung und danke Ihnen für Ihre Zeit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>9743</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Datenschutz im Kundenservice</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich erkundigen, ob Sie Datensicherheitslösungen für Gesundheitsanbieter und Krankenhaus-IT-Systeme anbieten. Können Sie detaillierte Informationen zu den Maßnahmen bereitstellen, die die Vertraulichkeit, Integrität und Verfügbarkeit sensibler Patientendaten sicherstellen? Ich würde auch gerne wissen, ob Sie Informationen zu etwaigen Compliance-Zertifizierungen wie HIPAA bereitstellen können. Zudem interessiere ich mich für den Incident-Response-Plan im Falle eines Sicherheitsverstoßes. Bitte stellen Sie relevante Dokumentationen und Referenzen aus vertrauenswürdigen Quellen zur Verfügung. Ich freue mich auf Ihre Rückmeldung. Vielen Dank für Ihre Zeit und Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>26497</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Software-Fehler und Abstürze bei Avast SQL Server</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Es treten Abstürze auf, wenn Avast SQL Server eingesetzt wird.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>18217</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Beim letzten Investitionsbericht gab es Rechnungsfehler aufgrund von Datenintegrationsschwierigkeiten und Softwarekonflikten. Die Zahlungsparameter wurden überprüft und die Softwareversionen aktualisiert, um das Problem zu beheben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>21403</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Hilfe Datenschutzverletzungen</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Es wurde eine mögliche Datenschutzverletzung in den IT-Systemen des Krankenhauses festgestellt, was die Sicherheit medizinischer Daten gefährdet hat. Anfangs wurden System-Scans durchgeführt und die Antivirus-Software aktualisiert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>22373</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Kundenservice, Datenanalysewerkzeug effizient Verarbeitung Investitionsdaten</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Kundenservice, Datenanalysewerkzeug effizient Verarbeitung Investitionsdaten eingesetzt. Fehler Kompatibilitätsprobleme Softwarebereich hinweisen. betroffenen Software- Geräte-Updates durchgeführt, Problem behält bestehen. Prüfung Datendatenquellenintegrität Identifizierung Grundursache vollem Gange. besorgt möglichen Auswirkungen Geschäft Unterstützung Lösung Angelegenheit frühen Zeitpunkt Anspruch nehmen. Bitte geben nächsten Schritte an, ergreifen können.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>12823</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, wir schreiben Ihnen, da wir ein ernstes Problem mit unserem IT-System des Krankenhauses festgestellt haben. Letztens wurde ein unerlaubter Zugangsantrag gestellt, der möglicherweise auf eine Software-Vulnerabilität zurückzuführen sein könnte. Um das Problem zu beheben, wurden sämtliche Sicherheitsprotokolle aktualisiert und Zugangspasswörter geändert. Trotz dieser Maßnahmen gibt es weiterhin Bedenken hinsichtlich der Sicherheit unserer medizinischen Daten. Wir schätzen Ihre Hilfe, um die Angelegenheit zu beleuchten und Rat einzuholen, wie wir unsere Systeme sichern können. Bitte informieren Sie uns darüber, welche Schritte wir unternehmen können, um zukünftige Unstimmigkeiten zu vermeiden. Wir freuen uns auf Ihre Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>20582</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Sicherheitsfall medizinischer Daten</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice,
+Wir haben einen Sicherheitsfall identifiziert, der potenziell auf unautorisierten Zugriff auf medizinische Daten zurückzuführen sein könnte. Dies lag an einer falsch konfigurierten Netzwerksicherheitsmauer. Bislang wurden die Zugriffsprotokolle geprüft, und Sicherheitsrichtlinien wurden vorübergehend verstärkt.
+Wir nehmen diesen Fall ernst und arbeiten daran, den Umfang des Falles zu bestimmen. Darüber hinaus überprüfen wir gründlich unsere Sicherheitsprozesse, um zukünftig ähnliche Fälle zu vermeiden.
+Bitte melden Sie sich bei Bedarf an, um weitere Informationen oder Unterstützung zu erhalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>14099</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Problem mit Marketing-Kampagnen</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Die digitale Marketingkampagne funktioniert nicht optimal unter neuen Algorithmen, was zu weniger Marke-Engagement und Wachstum führt. Die Werbelastung und die Zielgruppen sind ausgewogen, Verbesserung ist erforderlich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>22539</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Hilfe bei Investitionswerkzeug</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Investitionswerkzeug produziert ungenaue Berichte aufgrund von Softwarekonflikten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>20262</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Fragen zur Datenschutzmaßnahmen für Krankenhaus-IT-Lösungen</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Kontaktieren Sie mich bitte, um detaillierte Informationen über die Datenschutzmaßnahmen für Krankenhaus-IT-Lösungen zu erhalten. Interessiert sind wir insbesondere an den Protokollen, Technologien und Sicherheitsmechanismen, die dazu beitragen, vertrauliche Patientendaten zu schützen. Wir würden uns freuen, wenn Sie uns über verfügbare Schutzmaßnahmen wie Verschlüsselung, Zugriffskontrolle und die Einhaltung relevanter Vorschriften aufklären könnten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>22644</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Medizinische Datenschutzprobleme gemeldet</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>erleben unbefugten Zugriff auf medizinische Daten, möglicherweise veraltete Sicherheitsprotokolle. Neueste Softwareupdates könnten die Ursache sein. Stärkung der Feuergardenschutzeinstellungen und Passwörter aktualisieren, jedoch Schwachstellen feststellen. Unterstützung benötigt, um das Problem zu lösen und die Sicherheit unserer Daten zu gewährleisten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>13597</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Technische Sorge</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Es wurde ein Sicherheitsfall gemeldet, bei dem medizinische Daten im NAS-System und in MySQL-Datenbanken verunreinigt wurden. Dies könnte aufgrund von unzureichenden Zugriffssteuerungen und möglicherweise ausgelöst durch endgültig beendete Vulnerabilitäten passiert sein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>8248</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Bekümmernisse hinsichtlich der digitale Strategie der Marketing-Agentur sind in der Sichtbarkeit zu beklagen. Obwohl vorläufige Analysen auf schlechte Kampagnenzielgruppen hindeuteten und obwohl mehrere Strategien getestet wurden, zeigten sich erkennbare Verbesserungen des Engagements erst nach einigen Tagen. Derzeit erfolgt die aktuelle Prüfung der Kampagnendaten, um die Botschaft anzupassen und die Markenwahrnehmung sowie das Engagement zu verbessern. Ich möchte eine Diskussion einleiten und Ihnen empfehlen, uns anzurufen, um einen Fortschrittsbericht zu erhalten und mögliche nächsten Schritte zu besprechen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>13827</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Hilfe bei Sicherheitsproblemen</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Geliebte Kundenservice, ich schreibe, um eine Sicherheitsverletzung zu melden, die die medizinischen Daten des Krankenhauses beeinträchtigt hat. Es scheint, dass veraltete Sicherheitsprotokolle die Ursache sein könnten. Wir haben bereits Maßnahmen ergreifen können, wie das Aktualisieren der Passwörter, die Überprüfung der aktuellen Software auf mögliche Schwachstellen. Trotzdem wären wir dankbar für weitere Unterstützung bei der Untersuchung der Verletzung und der Umsetzung zusätzlicher Sicherheitsmaßnahmen, um zukünftige Verletzungen zu vermeiden. Könnten Sie bitte Ratschläge geben, wie wir dies am besten tun können?</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>12256</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Einbinden von Evernote SaaS</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Können Sie uns mehr Details zur Integration von Evernote in unser Projektmanagement-SaaS-System geben? Unsere Arbeitsgruppe würde sich freuen, operational Effizienz zu steigern, indem wir Evernote hinzufügen. Wir möchten gerne wissen, welche Schritte erforderlich sind, um Evernote in unserem System zu integrieren. Wir bedanken uns im Voraus für Ihre Unterstützung und freuen uns darauf, bald von Ihnen zu hören.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>7354</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Update des Abrechnungssystems</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte die Aktualisierung des Abrechnungssystems beantragen, um die Unterstützung für verschiedene Zahlungsmethoden bei betroffenen Produkten zu gewährleisten. Es ist wichtig, Sicherheits- und Funktionsverbesserungen mit hoher Priorität umzusetzen. Das derzeitige System ist veraltet und benötigt ein Upgrade. Wir hoffen auf eine zügige Bearbeitung unseres Anliegens und danken im Voraus für Ihre Unterstützung. Wir freuen uns auf eine baldige Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2899</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich nach Zahlungsoptionen und Zahlungsplänen für die Produkte Klipsch ProMedia 2.1 THX und Norton 360 erkundigen. Ich bin an einem Kauf interessiert und möchte mehr über die verfügbaren Zahlungsarten, Abrechnungszyklen sowie mögliche Rabatte und Aktionen erfahren. Könnten Sie bitte Informationen zu verschiedenen Bezahlmethoden, Zahlungsplänen sowie zu den Preisen, etwaigen Zusatzkosten und Paketangeboten mit Rabatten für den gemeinsamen Erwerb beider Produkte bereitstellen? Ich schätze Ihre Unterstützung sehr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>19593</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Schutz medizinischer Daten in Microsoft Office 365</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Liebe Kundensupport, Sie, erfahren, können Microsoft Office 365 in medizinischen IT-Umfeldern vertrauliche medizinische Daten sicherstellen? Bitte geben Sie Details zu besten Praktiken und Protokollen, die dafür sorgen, dass solche Informationen geheim, unveränderlich und verfügbar bleiben. Ich freue mich auf jegliche Anleitungen und Ressourcen, die zur Verfügung gestellt werden können. Danke für Ihre Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>5939</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Jenkins Marketing Automation Brand Growth Strategy</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Bitte stellen Sie Anweisungen zur Nutzung der Jenkins Marketing-Automatisierung bereit, um die Markenwachstumsstrategie zu optimieren und die Gesamtleistung zu steigern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>21799</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Integration von PostgreSQL - Unterstützung von Pluralsight</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Könnten Sie bitte mehr Informationen zur Integration von PostgreSQL liefern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>27870</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, ich würde gerne mehr über Lösungen zur Sicherung medizinischer Daten in Krankenhaus-IT-Systemen erfahren. Könnten Sie bitte mehr Informationen zu den Maßnahmen geben, die genommen werden, um sensible Patientendaten vor Cyberangriffen zu schützen? Ich freue mich darauf, weitere Details zu erhalten über Sicherheitsprotokolle und -technologien. Vielen Dank für Ihre Unterstützung. Ich freue mich darauf, bald von Ihnen zu hören.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>25313</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Aktualisierung von Express JS</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, ich möchte die Aktualisierung der Kompatibilität von Express.js in unserem Softwareprodukt für das Projektmanagement und unsere SaaS-Plattform bitten. Momentan verursacht die Integration Schwierigkeiten, da die aktuelle Version von Express.js veraltet ist. Ich schätze es, wenn Sie Anleitungen zur Aktualisierung von Express.js zur Verfügung stellen könnten, um eine glatte Integration in unser Softwareprodukt zu gewährleisten. Eine Aktualisierung ist für die Leistung und Sicherheit unserer Plattform von entscheidender Bedeutung. Bitte teilen Sie mich mit, wenn weitere Informationen erforderlich sind. Ich freue mich auf Ihre Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>5304</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>SaaS Outlook-Tools Integration Assistance</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Bitte stellen Sie eine Anleitung für den Integrationsprozess bereit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>9519</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte ein Problem beim Datenzugriff des Gesundheitsanbieters melden. Wir erleben Verzögerungen beim Zugriff auf Patientendaten, was unserer Ansicht nach auf Integrationsprobleme mit AWS, Elasticsearch und Zapier-Workflows zurückzuführen ist. Unser Team versucht, das Problem durch Neustart der Systeme und Löschen der Cache-Daten zu beheben, jedoch blieb das Problem bestehen. Wir befürchten, dass diese Schwierigkeiten die Fähigkeit beeinträchtigen könnten, Patienten rechtzeitig zu versorgen. Wir schätzen, wenn Sie die Angelegenheit dringend prüfen und eine möglichst schnelle Lösung anbieten könnten. Bitte lassen Sie uns wissen, wie wir weiter vorgehen sollen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>3879</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Anfrage zu Data Analytics Lösungen</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Sehr geehrtes Kundensupport-Team, ich möchte mich nach Data Analytics Lösungen zur Optimierung von Investitionsstrategien und Portfoliorenditen erkundigen. Könnten Sie bitte weitere Informationen zu den angebotenen Data Analytics Tools bereitstellen, beispielsweise prädiktives Modellieren, Risikoanalyse und Leistungskennzahlen? Ich würde mich auch freuen, wenn Sie Fallstudien und Erfolgsgeschichten früherer Kunden teilen könnten, die Data Analytics Lösungen genutzt haben, um ihre Investmentergebnisse zu verbessern. Zusätzlich bitte ich um Informationen zum Implementierungsprozess, inklusive etwaiger Schulungen und Unterstützung für das Team. Ich bin interessiert an maßgeschneiderten Lösungen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>1128</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Sicherheitsproblem bei Daten</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Ein Gesundheitsdienstleister hat eine potenzielle Datenverletzung erkannt, die medizinische Aufzeichnungen aufgrund veralteter Sicherheitsmaßnahmen betrifft. Erste Software-Updates wurden bereits durchgeführt, jedoch ist das Problem noch nicht vollständig behoben. Weitere Untersuchungen und Updates sind notwendig, um die Sicherheit sensibler Patientendaten zu gewährleisten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>17586</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Probleme mit Software-Abstürzen</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Es treten Abstürze bei Avast und SQL Server auf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>9686</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Anfrage zu Digital Marketing Markenentwicklungsstrategien</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich nach den Abrechnungsinformationen und Zahlungsmöglichkeiten für Dienstleistungen im Bereich Digital Marketing und Markenwachstum erkundigen. Könnten Sie mir bitte weitere Details zu den verfügbaren Plänen und deren jeweiligen Preisen zusenden? Ich bin daran interessiert, mehr darüber zu erfahren, wie Ihre Dienstleistungen Unternehmen beim Wachstum und Erfolg im digitalen Umfeld unterstützen können. Vielen Dank im Voraus für Ihre Zeit und Unterstützung. Ich freue mich auf Ihre baldige Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>20726</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Plötzlicher Abfall der Beteiligungsmetriken für die Kampagne</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Wir haben einen plötzlichen Abfall der Beteiligungsmetriken bei unserer digitalen Kampagne beobachtet. Dies scheint mit den neuesten Änderungen an den Suchmaschinennutzeralgorithmen zusammenhängen zu können. Wir haben versucht, unser Werbemodell anzupassen und Inhalte zu aktualisieren, aber das Problem blieb bestehen. Könnten Sie bitte helfen, die Ursache zu ermitteln und einen Lösungsansatz zu finden, um die Beteiligungsmetriken zu verbessern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>14919</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Bewerbung für digitale Strategiedienstleistungen</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Ich bin interessiert, mehr über digitale Strategiedienstleistungen zu erfahren. Könnten Sie mehr Details geben? Insbesondere interessiert es mich, zu erfahren, ob diese Dienstleistungen die Markengröße fördern können. Die bereitgestellten Informationen, insbesondere zum Ansatz und den Vorteilen der Dienstleistungen, schätze ich sehr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>21116</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Campagne hatte Schwierigkeiten bei der Kundenkontaktaufnahme</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Die letzte Campagne scheiterte aufgrund technischer Probleme. Die Fehlerbehebung war erfolglos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>26134</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Bitten um Informationen zu API-Integrationsmöglichkeiten für Projektmanagement-Softwareas-a-Service (SaaS)</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice-Abteilung, könnten Sie bitte mehr Details zu verfügbaren APIs sowie deren Funktionalitäten und Unterstützungsmaterialien zur Verfügung stellen? Es wäre außerdem sehr hilfreich, Beispiele erfolgreicher Integrationsprojekte unserer Kunden zu erhalten. Diese Informationen würden mir einen besseren Überblick über die Möglichkeiten des Plattformangebots geben. Vielen Dank für Ihre Zeit und Unterstützung. Ich freue mich darauf, bald von Ihnen zu hören. freundliche Grüße, [Ihr Name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>7553</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte eine Aktualisierung der Produktintegrationskompatibilität anfragen. Es geht um die genannten Software- und Hardware-Komponenten sowie um die erweiterte SaaS-Skalierbarkeit. Die derzeitige Integration ist veraltet und verursacht Schwierigkeiten im Arbeitsablauf. Daher bitte ich, die Integration auf die neueste Version zu aktualisieren, um eine reibungslose Kompatibilität zu gewährleisten. Ein Update würde unserem Team ermöglichen, effizienter und effektiver zu arbeiten. Wir würden eine schnelle Bearbeitung und eine Lösung sehr schätzen. Vielen Dank für Ihre Zeit und Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>24143</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Bewerber von Kundenservice, um Informationen zur Optimierung der Investitionen in Apache Hadoop und Datenaufbereitung zu erhalten. Bitte mehr Details liefern, um die Unterstützung zu verbessern.</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich bitte um Informationen zur Optimierung von Investitionen in Apache Hadoop sowie zur Datenaufbereitung. Könnten Sie mir mehr Details liefern, um die Unterstützung weiter zu verbessern? Ich freue mich auf Ihre Informationen und Ressourcen. Vielen Dank für Ihre Unterstützung und freue mich darauf, bald eine Rückmeldung zu erhalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>3846</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Probleme mit der Synchronisierung mehrerer Produkte</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Betroffene Benutzer beklagen sich von häufigen Synchronisationsproblemen bei verschiedenen Produkten, was die Projektaktualisierungen und Kooperation beeinträchtigt. Mögliche Gründe könnten ein Serverüberlastungsproblem, Integrationsprobleme oder Datenungleichgewichte sein. Verschiedene Maßnahmen, wie Neustarten der betroffenen Dienste, Leerstellen der Caches und Überprüfung der Serverprotokolle, wurden bereits unternommen, aber das Problem behält sich bestehen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>8516</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Sicherheitsverletzung im Krankenhaussystem</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Das IT-System des Krankenhauses wurde Opfer einer Sicherheitsverletzung, insbesondere im Bereich der medizinischen Daten und Gerätesicherheit. Vermutlich liegt das Problem an veralteten Sicherheitsprotokollen. Die Passwörter wurden zurückgesetzt, und ein erster Virenscan wurde durchgeführt, um das Problem zu beheben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>20233</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Datenanalyse für Investitionsdienstleistungen</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Ich bin interessiert, mehr über Datenanalyse-Dienstleistungen und deren Optimierung Investitionsstrategien zu erfahren. Ich würde gerne mehr Informationen über die verwendeten Tools und Techniken, und wie diese helfen können, informierte Entscheidungen zu treffen. Ich freue mich auf Ihre Rückmeldung und freue mich darauf, zusätzliche Details zu erhalten. Bitte geben Sie mir eine Möglichkeit, mich zu kontaktieren, um diese Dienstleistungen besprechen zu können.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>6531</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Anfrage zur Abrechnung von Marketingdienstleistungen</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich nach den verfügbaren Zahlungsplänen für Marketingdienstleistungen im Zusammenhang mit den aufgeführten Produkten erkundigen. Könnten Sie bitte eine detaillierte Aufschlüsselung der verbundenen Kosten bereitstellen, einschließlich möglicher Rabatte oder Aktionen, die verfügbar sein könnten? Ich bin daran interessiert, die verschiedenen Marketingkanäle zu erkunden, die Ihr Unternehmen anbietet, wie z.B. Social-Media-Werbung, E-Mail-Marketing und Suchmaschinenoptimierung. Zudem möchte ich mehr über die Preisstruktur der Dienste erfahren, um die zu erwartenden Ergebnisse besser einschätzen zu können. Zusätzlich bitte ich um Informationen zu Einrichtungsgebühren und laufenden Kosten der Dienste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>6161</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Zoho Books Integration mit Projektmanagement-Plattform</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte anfragen, ob eine Integration der Zoho Books SaaS-Projektmanagementplattform möglich ist. Könnten Sie bitte ausführliche Dokumentationen und Anleitungen bereitstellen, um die Integration erfolgreich durchzuführen? Ich benötige Informationen zu den erforderlichen Schritten, den notwendigen Zugangsdaten sowie möglichen Einschränkungen. Da die Integration für unsere Geschäftsprozesse von großer Bedeutung ist, freue ich mich auf eine zeitnahe Rückmeldung. Bitte informieren Sie mich auch, ob zusätzliche Ressourcen oder Unterstützung verfügbar sind, um einen reibungslosen Integrationsprozess sicherzustellen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>13684</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Bitten Sie um Informationen zur Integration von Khan Academy Projektmanagement-Software-as-a-Service</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Ich möchte mich bei Ihnen melden, um zu erkunden, ob es möglich ist, Khan Academy Projektmanagement-Software-as-a-Service in unser System einzubinden. Könnten Sie mir mehr Details zu den Vorteilen und wie die Integration die Projektmanagement-Erfahrung verbessern kann, geben? Ich würde Ihre detaillierten Erklärungen sehr schätzen. Vielen Dank für Ihre Unterstützung. Ich freue mich darauf, von Ihrer Antwort zu hören.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>4829</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte Sie darüber informieren, dass unser Gesundheitsdienstleister ungewöhnliche Zugriffsversuche auf medizinische Daten festgestellt hat, was auf einen Phishing-Angriff hindeuten könnte. Unsere erste Reaktion bestand darin, die Firewall-Regeln zu aktualisieren und die Überwachung zu verstärken. Glücklicherweise wurden bisher keine Datenverletzungen festgestellt. Wir nehmen die Angelegenheit sehr ernst und arbeiten daran, die Sicherheit unserer Systeme zu gewährleisten. Wir werden Sie über weitere Entwicklungen auf dem Laufenden halten. Bitte lassen Sie uns wissen, falls Sie Fragen oder Bedenken haben. Wir schätzen Ihre Aufmerksamkeit in dieser Angelegenheit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>14206</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Datensperrverstoß gemeldet</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, ich melde euch einen schweren Fehler. Unverschlüsseltes Zugriff auf sensiblen medizinischen Daten wurde ermöglicht, was auf alten Software-Sicherheitslücken zurückzuführen ist. Trotz der Sicherheitsprotokoll-aktualisierung sind Sperrverstöße weiterhin in verschiedenen Systemen und Geräten zu beobachten. Dieser Datensperrverstoß bedroht vertrauliche Patientendaten und könnte zu Konsequenzen führen. Ich bitte um sofortige Behandlung der Angelegenheit, um weitere Sperrverstöße zu verhindern. Bitte untersucht die Angelegenheit und gebt eine Lösung, um die Systeme sicherer zu machen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>13403</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Hilfe bei Systemstörungen</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Kürzlich gab es mehrere Systemstörungen, die die Leistung mehrerer Anwendungen beeinträchtigten und Investitionsanalyseprozesse verzögerten. Das Problem scheint auf Konflikten zwischen konfliktierenden Softwareupdates und Installationsprozessen zurückzuführen. Ich habe bereits versucht, die betroffenen Anwendungen neu zu starten und nach den neuesten Updates zu suchen, aber die Probleme bestehen leider immer noch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>18934</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Probleme mitlangsamen Ladens Projektmanagement-Plattform</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Beobachtet langsamen Ladeprozess bei der Projektmanagement-Plattform.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>19613</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Sichere Verwaltung medizinischer Daten in MongoDB</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Könnten zusätzliche Details zur Sicherung medizinischer Daten in MongoDB 4.4 für IT-Abteilungen von Krankenhäusern bereitstellen, um die besten Praktiken und Vorschriften zu erfüllen? Ich suche nach einem sicheren System, das Anweisungen bietet. Vielen Dank für Ihre Unterstützung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>9244</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Gesundheitsdaten-Schutz und IT-Services in Krankenhäusern</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Ich möchte mich erkundigen, welche Lösungen im Bereich Sicherheit und Datenschutz für Gesundheitsdaten durch IT-Dienstleistungen in Krankenhäusern angeboten werden. Können Sie detaillierte Informationen über die verfügbaren Dienste bereitstellen? Besonders interessiert bin ich an Sicherheitsmaßnahmen zum Schutz sensibler Patientendaten. Zudem hätte ich gern Informationen zu den IT-Services für Krankenhäuser, einschließlich etwaiger Software- und Hardwarelösungen. Bitte fügen Sie auch relevante Preis- und Paketdetails bei. Ich freue mich auf Ihre Rückmeldung und darauf, mehr über Ihre Dienstleistungen zu erfahren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>7559</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Probleme bei Digitalen Kampagnen</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte meine Bedenken hinsichtlich der kürzlich durchgeführten digitalen Kampagnen unserer Marketingagentur äußern. Leider haben die Kampagnen nur durchschnittliche Ergebnisse erzielt, und ich habe Schwierigkeiten, die Ursachen dafür zu verstehen. Erste Analysen deuten auf ineffizientes Targeting und Plattformprobleme hin, die möglicherweise die Leistung beeinträchtigen. Trotz Anpassungen bei den Anzeigenformaten und den Budgets wurden keine signifikanten Verbesserungen festgestellt. Ich würde es schätzen, wenn Sie die Angelegenheit prüfen und Ratschläge geben könnten, wie wir die digitalen Kampagnen optimieren können, um bessere Resultate zu erzielen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>15236</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Kontaktieren Sie uns, um mehr über digitale Strategien zur Förderung des Markenwachstums zu erfahren. Könnten Sie Details zu den Methoden erhalten, die die Markenbewusstheit und die Nachhaltigkeit der Kunden steigern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>15179</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Problem Mit Datenzugriff</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Lieber Kundenservice, wir begegnen unerwarteten Datenzugriffsproblemen im Gesundheitsinformationssystem. Es könnte sich auf mögliche falsche RAID-Konfigurationen beziehen. Nachdem wir den RAID-Controller für die verbundenen Geräte, einschließlich Crucial MX500 SSDs, zurückgesetzt haben, behält das Problem weiterhin an. Das Team hat verschiedene Schritte zur Problemlösung unternommen, aber das Problem konnte noch nicht gelöst werden. Wir schätzen Ihre Unterstützung bei der Identifikation der Ursache, um eine Lösung bereitzustellen und das System einwandfrei zu betreiben. Bitte teilen Sie uns mit, falls weitere Informationen erforderlich sind. Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>1300</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Schutz medizinischer Informationen</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Benötige Hinweise zur Sicherung medizinischer Daten bei der Integration von QuickBooks Online mit Airtable für Abrechnungen im Gesundheitswesen. Können Schritt-für-Schritt-Anleitungen bereitgestellt werden?</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>22839</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Sicherung medizinischer Daten in Krankenhäusern mit Kaspersky Internet Security 2021</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Ich möchte erfahren, wie Kaspersky Internet Security 2021 zur Sicherung medizinischer Daten in Krankenhäusern eingesetzt werden kann. Könnten Sie bitte Details zu dem Lösungsansatz geben?</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>22267</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Medizinischer Datenschutzverstoß</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Es wurden mehrere Fälle unerlaubten Zugriffs auf medizinische Daten gemeldet, was die patientschützende Geheimhaltung gefährdet. Mögliche Gründe umfassen fehlende IT-Sicherheitsprotokolle, mangelnde Mitarbeiterbildung und fragwürdige Datensicherheitsmaßnahmen. Um das Problem zu lösen, wurden sofortige Software-Updates und eine Überprüfung bestehender Sicherheitsmaßnahmen durchgeführt, um zukünftige Vorfälle zu vermeiden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>6407</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Anfrage zu Skalierbarkeitsfunktionen und Testoptionen</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Ich bin daran interessiert, mehr über die Skalierbarkeitsfunktionen unseres SaaS-Angebots zu erfahren. Könnten Sie bitte Details dazu bereitstellen, wie die Plattform zunehmenden Traffic bewältigt? Gibt es Testmöglichkeiten, bei denen der Service in einer kostenpflichtigen Version ausprobiert werden kann? Ich schätze Informationen über Skalierbarkeits-Tests und deren Möglichkeiten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>27738</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Hilfe bei der Entwicklung einer digitalen Markenwachstumsstrategie</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Möchten Sie Details zu Informationen, die die Förderung des Markenwachstums durch digitale Strategien unterstützen können? Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>9855</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Support-Anfrage für Sage Accounting</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundendienst, ich möchte mich erkundigen, ob die Sage Accounting Projektmanagement-SaaS-Plattform integriert werden kann. Könnten Sie bitte detaillierte Dokumentationen zum Ablauf bereitstellen? Eine Anleitung mit Ressourcen würde den Einstieg erleichtern. Vielen Dank im Voraus für Ihre Unterstützung. Ich freue mich auf Ihre Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>25297</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Verbesserung Investitionen AWS Analytics</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, bitten Sie, nachzufragen, ob Sie Rat geben können, wie Investitionen in AWS Alteryx für Datenanalyse optimiert werden können. Würden Sie Ratschläge geben, wie bestimmte Werkzeuge verwendet werden können, um informierte Investitionsentscheidungen zu treffen? Es wäre von Interesse, mehr über die Fähigkeiten von AWS Alteryx zu erfahren, wie sie integriert werden können, um große Datensätze zu analysieren, Trends zu identifizieren und Investitionsportfolios zu optimieren. Ich freue mich, über dieses Thema weitere Informationen zu erhalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>1319</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Investitionsanalyse Plattform - Verzögerungen bei Datenverarbeitung</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Die Investitionsanalyseplattform unseres Unternehmens hat Verzögerungen bei der Datenverarbeitung erlebt, wahrscheinlich infolge kürzlicher Software-Updates. Erste Maßnahmen zur Fehlerbehebung umfassten den Neustart des Systems sowie Datenvalidierungsprüfungen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>11537</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Interrhythmische iOS-Verbindungsprobleme bei SaaS-Projektmanagement-Tool gemeldet</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Nutzer erleben Intermittierende Verbindungsprobleme mit dem SaaS-Projektmanagement-Tool auf iOS-Geräten. Trotz Neustarts des Routers und Anpassung der Anwendungs-Einstellungen bestehen die Probleme weiterhin. Es wird vermutet, dass die Probleme auf die Router-Konfiguration oder die WLAN-Router-Kompatibilität zurückzuführen sind. Bitte helfen Sie dabei, das Problem zu beheben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>25492</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Forderung integrierte Funktionen PrestaShop Shopware</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Ich interessiere mich für mehr integrierte Funktionen der Software-as-a-Service-Lösung PrestaShop Shopware. Könnten Sie bitte mehr Informationen zur Verfügbarkeit von Integrationsfunktionen, insbesondere zur Datensynchronisierung und Bestellverwaltung, zur Verfügung stellen? Es wäre schön, wenn Sie jegliche Dokumentation oder Tutorials zur Verfügung stellen könnten, die mir helfen, den Integrationsprozess zu beginnen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>25567</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Potentielle Sicherheitslücke in Krankenhaus-Systemen</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Es wurde eine potenzielle Sicherheitslücke in den IT-Systemen des Krankenhauses festgestellt, die sich aus einer Software-Verzugsfalle ergeben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>23034</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Datensperrungsfall bei Gesundheitsdiensten</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Lieber Kundenservice, ein potenzielles Datensperrungsverfahren hat bei Gesundheitsdiensten zu Problemen bei sensiblen medizinischen Daten bei Krankenhäusern geführt. Die Ursache könnte ein veraltetes Sicherheitsprotokoll oder eine fehlerhafte Firewall-Konfiguration sein. Wir versuchen, die Sicherheitssoftware zu aktualisieren und das Netzwerkverkehr zu überwachen, aber die Probleme blieben bestehen. Bitte untersuchen Sie die Angelegenheit sofort, um die Integrität unserer Systeme zu gewährleisten. Wir bedanken uns für Ihre umgehende Aufmerksamkeit auf diesem dringenden Thema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>27687</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Optimierung der Datensicherheit im Medizinischen Bereich</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, ich schreibe Ihnen mit Bezug zur Verbesserung der Datensicherheitsmaßnahmen, insbesondere im Schutz von medizinischen Informationen in den IT-Systemen von Krankenhäusern. Da die Vertraulichkeit und Sensitivität dieser Informationen von hoher Bedeutung ist, ist es entscheidend, die notwendigen Maßnahmen zu treffen, um unautorisierten Zugriff und Datenverletzungen zu verhindern. Bitte setzen Sie zusätzliche Sicherheitsprotokolle wie Verschlüsselung, Firewalls und Zugriffssteuerungen um, um die medizinischen Informationen zu schützen. Darüber hinaus sollten regelmäßige Sicherheitsprüfungen und Trainings durchgeführt werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>14602</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Optimierung finanzieller Analysen mit Oracle Database 19c</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Ich schreibe, um tiefergehende Erkenntnisse zu gewinnen und zu erfahren, wie Oracle Database 19c für die finanzielle Datenanalyse und Investitionsoptimierung eingesetzt werden kann. Es wäre hilfreich, Anleitungen und Informationen zu den besten Praktiken für die Verwendung verfügbaren Werkzeuge zum datengetriebenen Entscheidungsprozess in der Finanzbranche zu erhalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>4461</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Benötigte Unterstützung im Marketingbereich</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich schreibe, um auf die geringe Beteiligung aufmerksam zu machen, die die letzte digitale Kampagne unserer Marketingagentur gezeigt hat. Es besteht der Verdacht, dass unsere Zielstrategien veraltet sind, was möglicherweise zu mangelndem Interesse bei unserer Zielgruppe führt. Es wurden bereits Anstrengungen unternommen, um die Anzeigen zu optimieren, doch leider haben diese nur minimale Verbesserungen erbracht. Ich bin besorgt, dass dies die Sichtbarkeit unserer Marke und unsere Umsätze negativ beeinflussen könnte. Wir schätzen Ihre Unterstützung und Empfehlungen sehr, um die Zielstrategien neu zu gestalten und die Beteiligung zu erhöhen. Bitte lassen Sie uns wissen, wie Sie uns dabei unterstützen können.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>7982</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Anfrage zu digitalen Strategien für das Markenwachstum</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich erkundigen, welche digitalen Strategien Ihre Marketingagentur für das Wachstum einer Marke anbietet. Könnten Sie bitte detaillierte Anweisungen geben, wie Ihre Agentur Unternehmen dabei unterstützen kann, ihre Online-Präsenz zu erweitern und die Markenbekanntheit zu steigern? Besonders interessieren mich die Arten der Dienstleistungen, die angeboten werden, wie beispielsweise Social-Media-Management, Content-Erstellung und Suchmaschinenoptimierung. Außerdem hätte ich gerne Informationen zu den Kosten, der Dauer und den Details der Dienstleistungen. Vielen Dank im Voraus für Ihre Unterstützung. Ich freue mich auf Ihre baldige Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>26587</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Fehler bei Tracking-Werkzeugen</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Es tut uns leid, dass Sie Probleme mit den Tracking-Werkzeugen haben. Bitte geben Sie mehr Informationen zu Ihrem Problem, einschließlich eines Beispiels, wenn möglich, der spezifischen Werkzeug und der Fehlermeldung, die Sie erhalten haben. Dies wird uns helfen, eine bessere Lösung für Ihr Problem zu finden. Sie können sich auch an die Nummer &lt;tel_num&gt; wenden, um die Diskussion fortzusetzen, falls dies nötig ist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>26361</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Bitten um Ausführlichere Informationen zu Anlagenerhöhungsdienstleistungen und Datenanalyselösungen</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Könnten Sie mir bitte mehr Informationen zu Anlagenerhöhungsdienstleistungen und Datenanalyselösungen geben? Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>25667</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Anfrage an Kundendienst</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Könnten mehr Details über digitale Strategien gegeben werden, um das Markenwachstum zu fördern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>15135</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, 
+ein potentieller Datenverlust wurde im medizinischen IT-System festgestellt, die Vertraulichkeit medizinischer Akten wurde gefährdet. Dies scheint auf veraltete Software und Schwachstellen zurückzuführen sein. Vorübergehende Sicherheitspatches wurden implementiert, die Antivirus-Software wurde aktualisiert, trotzdem bestehen Befürchtungen. 
+Der Datenverlust umfasst sensible Patientendaten wie Namen, Adressen und medizinische Aktenverläufe. Wir nehmen dieses Thema ernst und benötigen Unterstützung für eine gründliche Untersuchung und die Implementierung zusätzlicher Sicherheitsmaßnahmen, um zukünftige Vorfälle zu verhindern. 
+Wir</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>26384</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Hilfe zur Entwicklung digitaler Wachstumsmethoden erforderlich</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice-Abteilung,
+Jeweils unsere Produkte auf digitalen Plattformen schlecht positioniert, was zu einer reduzierten Markenpräsenz und geringem Engagement führt. Die Ursachen scheinen ineffektiven Marketingstrategien und mangelnden SEO-Praktiken zu sein. Soziale Medien-Kampagnen und Websiteoptimierungen wurden durchgeführt, jedoch ohne die erwarteten Verbesserungen. Wir benötigen dringend Unterstützung, um unsere digitalen Wachstumsmethoden zu verbessern und unsere Onlinepräsenz zu optimieren. Das Team hat verschiedene Ansätze versucht, jedoch konnten die gewünschten Ergebnisse nicht erreicht werden. Wir würden die Anleitung und Empfehlungen schätzen, die uns helfen können, unsere Herausforderungen zu bewältigen und die Markenpräsenz zu erhöhen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>5065</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Schutz medizinischer Daten durch KNIME-Integration</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich bitte um Informationen zur Sicherung medizinischer Daten bei der Verwendung von KNIME im Rahmen bewährter Praktiken der Krankenhaus-IT-Integration. Könnten Sie eine Anleitung bereitstellen, um die Vertraulichkeit, Integrität und Verfügbarkeit sensibler medizinischer Informationen zu gewährleisten? Ich freue mich auf Empfehlungen zur Umsetzung robuster Sicherheitsmaßnahmen wie Verschlüsselung, Zugriffskontrollen und Audits. Außerdem interessiere ich mich für die Integration von KNIME in Krankenhaus-IT-Systeme, einschließlich elektronischer Gesundheitsakten und Laborsystemen. Bitte stellen Sie relevante Dokumentationen, Fallstudien und Beispiele zur Verfügung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>27336</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Verbesserte Sicherheitsmaßnahmen im Bereich medizinischer Datenschutz</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Ich schreibe an, um Verbesserungen in den Sicherheitsmaßnahmen und Datenschutz in der Medizin zu erörtern. Das Unternehmen plant, bestehende IT-Infrastrukturen mit Softwarelösungen zu integrieren, um die Vertraulichkeit, Integrität und Verfügbarkeit sensibler medizinischer Informationen zu sichern. Wir möchten mehr über die besten Praktiken in dieser Sache erfahren, um unser Ziel zu erreichen. Insbesondere interessieren uns Kryptografiemethoden und Zugriffssteuerungen, um medizinische Daten zu schützen. Wir glauben, dass die Steigerung der Sicherheitsmaßnahmen entscheidend ist, um das Vertrauen der Patienten aufrechtzuerhalten und den gesetzlichen Anforderungen gerecht zu werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>25395</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Anfragen zur Einholung von Kundendienst-Anleitungen für die Sicherung medizinischer Daten sowie Rücksichtnehmende Empfehlungen für Figma und Apple Xcode 12.5</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Ich würde gerne Informationen zu besten Praktiken und Sicherheitsmaßnahmen für die Verwaltung vertraulicher medizinischer Daten erhalten. Könnten Sie mir Rücksichtnehmende Empfehlungen für die Nutzung von Figma und Apple Xcode 12.5 zur Verfügung stellen? Ich freue mich auf Ihre Rückmeldung und freue mich darauf, Sie zu einem geeigneten Zeitpunkt kontaktieren zu können, um diese Themen zu besprechen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>16260</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, 
+es wurde eine potenzielle Datenverletzung in den Krankenhaus-IT-Systemen festgestellt, die klinische Akten gefährdet hat. Diese Schwachstellen sind wahrscheinlich auf veraltete Software zurückzuführen, obwohl bereits Anfangssicherheitspatches installiert wurden und die Antivirensoftware aktualisiert wurde. Trotzdem bestehen weiterhin Bedenken. 
+Die Verletzung hat sensible Patientendaten wie Namen, Adressen und medizinische Verlaufsuntersuchungen preisgegeben. Wir nehmen diesen Fall sehr ernst und wären dankbar für Unterstützung bei der Durchführung einer gründlichen Untersuchung und der Einführung zusätzlicher Sicherheitsmaßnahmen, um zukünftige Vorfall zu vermeiden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>15936</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>kommunizieren Sie, um mehr über SaaS-Features wie Projektmanagement und Skalierbarkeit zu erfahren. Könnten Sie detailliertere Informationen zu den Werkzeugen und Funktionen, die große Projekte und Teams unterstützen, geben? Ich freue mich auf eine effiziente Zusammenarbeit und die Diskussion von Aufgabenverwaltung. Danke für Ihre Unterstützung und freue mich auf Ihre Rückmeldung baldigst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>25854</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, bitten Sie, die Integration von TensorFlow in unsere Projektmanagement-Software zu berichten. Würden Sie gerne Details zur Integration sowie verfügbare Leitfäden und Tutorien bereitstellen? ich freue mich auf Informationen zu Anfangsschritten sowie möglichen Vorteilen und Einschränkungen bei der Nutzung der TensorFlow-Software. Vielen Dank für Ihre Unterstützung und freue mich auf Ihre baldige Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>7165</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr"/>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundendienst, ich möchte eine Aktualisierung unserer Data-Analytics-Tools beantragen, um die Investitionsplanung und die Genauigkeit der Berichterstattung unseres Finanzunternehmens zu verbessern. Das derzeitige System ist veraltet und behindert unsere Fähigkeit, fundierte Entscheidungen zu treffen. Wir benötigen fortschrittlichere Funktionen wie Echtzeit-Datenüberwachung, prädiktive Analysen und anpassbare Berichte. Ein Update würde es uns ermöglichen, unsere Kunden besser zu bedienen und im Wettbewerb zu bestehen. Wir würden es schätzen, wenn Sie uns einen Zeitplan und eine Kostenschätzung für die Aktualisierung zukommen lassen könnten. Vielen Dank für Ihre schnelle Aufmerksamkeit in dieser Angelegenheit. Ich freue mich auf Ihre Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>26015</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Optimierung des Kundensupports durch digitale Strategien</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundensupport-Abteilung, ich schreibe Ihnen, um die Umsetzung der überarbeiteten digitalen Strategien zu besprechen. Ziel ist es, die Markengröße zu stärken, die Nutzung verschiedener Plattformen zu verbessern und Online-Präsenz zu erhöhen. Dies umfasst die Nutzung von Social-Media-Beiträgen, E-Mail-Marketing-Kampagnen und Content-Creations-Verfahrensweisen. Wir möchten eine stärkere Verbindung zum Zielpublikum aufbauen und die Website-Besucherzahlen steigern, um unsere Geschäftsziele und Kundenerwartungen zu übertrumpfen. Ich freue mich darauf, Möglichkeiten zu finden, um unsere Marke online zu verbessern. Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>28222</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Problem mit Investment-Rückgangsanalyse</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Das Analysewerkzeug bietet unkonsequente Prognosen. Das Team hat die aktuellen Daten geprüft und versucht, die Modelle neu zu kalibrieren. Dies führte zum Erfolg. Wir benötigen Unterstützung, um das Problem zu lösen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>26796</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Verbesserung der Markensichtbarkeit online durch Effizienzverbesserungen</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundensupport, bitte überprüfen Sie, ob wir das Potenzial nutzen können, unsere Markensichtbarkeit mit Squarespace zu verbessern. Wir möchten unsere Online-Präsenz erweitern und freuen uns auf Tipps zu den besten Praktiken, wie Sie mit Squarespace Markensichtbarkeit erhöhen können. Besonders interessiert uns die Optimierung unserer Websites für Suchmaschinen und die Nutzung von Sozialmedien zur Vertrafbringerung und Anziehung von Verkehr auf unsere Seite. Vielen Dank für Ihre Geduld und Unterstützung. Wir freuen uns darauf, bald von Ihnen zu hören.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>8215</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Sicherheitsvorfallmeldung</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Der Gesundheitsdienstleister hat eine Sicherheitsverletzung erlebt, bei der medizinische Daten auf den IT-Systemen des Krankenhauses kompromittiert wurden. Mögliche Ursachen könnten kürzliche Software-Updates oder Phishing-Angriffe sein. Die ergriffenen Maßnahmen umfassen das Ändern von Passwörtern sowie das Durchführen von Antiviren-Scans. Der Vorfall hat erhebliche Störungen in der Patientenversorgung und im Krankenhausbetrieb verursacht. Eine Untersuchung ist im Gange, um die Ursache und das Ausmaß der Verletzung zu ermitteln. Vorübergehend sind Patienten aufgerufen, ihre persönlichen medizinischen Informationen aufmerksam zu überwachen und auf verdächtige Aktivitäten zu achten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>11591</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Funktionen API-Integration für Projektmanagement</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Guten Tag Kundenservice, ich wende mich an Sie, um mehr über API-Integration-Funktionen zu erfahren, die unsere Projektmanagementdienstleistungen skalieren können. Wir möchten unser aktuelles System erweitern und mehr über die API-Fähigkeiten erfahren. Könnten Sie uns mehr Informationen zu den integrierten Funktionen, wie zum Beispiel Datenabgleich und Workflowautomatisierung, geben? Darüber hinaus interessieren wir uns für besondere Einschränkungen hinsichtlich der Anzahl von Nutzern und Projekte, die durch die API verwaltet werden können? Wir freuen uns auf Ihre Rückmeldung mit weiteren Details.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>5999</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Datenschutzverletzung beim medizinischen Dienst durch veraltete Software</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Der medizinische Dienstleister hat eine Datenschutzverletzung erfahren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>24197</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Beratung zur Xero-Investment-Analyse</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundenservice, ich möchte mich mit der Nutzung von Xero für die Optimierung meiner Investments befassen. Könnten Sie mir Hinweise geben, wie ich den Einsatz des Systems optimal gestalten kann? Ich freue mich auf Ressourcen, Tipps und Unterstützung, die mir dabei helfen, meine Aufgabe erfolgreich umzusetzen. Vielen Dank für Ihre Unterstützung und freue mich auf eine baldige Rückmeldung von Ihnen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>9016</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Fehlerbericht im System</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Das Data-Analytics-System ist abgestürzt, was die Investitionsoptimierung behindert hat. Wahrscheinliche Ursache: Softwareinkompatibilität oder Überlastung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>20197</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr"/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>geehrte Kundenservice, ich schreibe Ihnen, um einen Fehler in der Projektmanagement-Software zu melden. Es tritt unter Umständen zeitweise ein Ausfall auf, was möglicherweise auf Serverbelastung oder Netzwerkprobleme zurückzuführen ist. Trotz unserer Bemühungen, die Server zu optimieren und die Ressourcenanzahl zu erhöhen, bleibt das Problem bestehen. Wir haben vermutet, dass eine schnelle Lösung möglich sein könnte, sobald die Untersuchung abgeschlossen ist. Wenn Sie weitere Informationen benötigen, um die Untersuchung durchzuführen, bitten wir Sie, uns zu informieren. Ich werde gerne bereitstehen, um die notwendigen Besprechungen zu organisieren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>9650</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Die digitale Strategie der Marketing-Agentur könnte positive Auswirkungen auf die Marke haben. Obwohl die vorläufige Analyse auf schlechte Kampagnenbezeichnungen schließen ließ, zeigten mehrere getestete Strategien sichtbare Verbesserungen in Bezug auf das Engagement. Derzeit wird die Kampagnendatenanalyse fortgesetzt und die Mitteilungsstrategie angepasst, um die Markebenennbarkeit und das Engagement zu verbessern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>28261</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Sicherheitslücke in KI-Systemen der Klinik</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Es wurde eine Sicherheitslücke in den KI-Systemen der Klinik festgestellt, was die Vertraulichkeit medizinischer Daten gefährdet. Wir haben versucht, das Software-Update durchzuführen und Sicherheitsmaßnahmen zu stärken, jedoch bestehen weiterhin Probleme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>17372</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Versicherung medizinischer Daten im Gesundheitswesen</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Betreff: Kundendienst, Kontakt bezüglich Sicherheitsmaßnahmen, Schutz medizinischer Daten in der Nutzung von Zapier und Zoho CRM in der Gesundheitsinformatik. Es ist wichtig, dass Gesundheitsorganisationen vertrauliche Patientendaten sicher verwahren und speichern. Ich interessiere mich für weitere Verschlüsselungsverfahren und die Compliance-Zertifizierungen, die Zapier und Zoho CRM erworben haben, z.B. HIPAA. Darüber hinaus brauche ich Informationen zu den Sicherheits-Einstellungen, Konfigurationen und Werkzeugen, die speziell für die strengen Sicherheitsstandards der Gesundheitsindustrie eingerichtet wurden. Könnten Sie einen Anruf vereinbaren, um detaillierte Informationen zu den Sicherheitsmaßnahmen und Compliance-Zertifizierungen zu besprechen?</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>6305</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Marketing-Kampagne funktioniert nicht optimal</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Die digitalen Strategien des Markenagents haben die Markensichtbarkeit reduziert. Mehrere Kampagnen wurden gestartet, aber die Ergebnisse sind schlecht. Es ist wahrscheinlich die ineffektive Zielgruppensegmentierung, die den Grund für diese Probleme bildet. Ich benötige Unterstützung, um die Onlinepräsenz des Markens zu verbessern und bessere Ergebnisse bei den Marketinganstrengungen zu erzielen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>8054</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Problem bei der Integration von Finanzdaten</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Das Finanzunternehmen erlebte ungenaue Resultate bei Investmentanalysen, vermutlich verursacht durch Fehler in der Datenintegration über mehrere Softwareplattformen hinweg. Die erste Problemlösung umfasste die Datenvalidierung und Kompatibilitätsprüfungen der Software, doch die Schwierigkeiten bestehen weiterhin. Die Fehler in der Datenintegration haben zu falschen Investmentempfehlungen geführt, was potenziell erhebliche finanzielle Verluste nach sich ziehen könnte. Um das Problem zu beheben, ist eine gründliche Überprüfung des Datenintegrationsprozesses sowie der Softwarekompatibilität notwendig. Es ist erforderlich, mit den Softwareanbietern zusammenzuarbeiten, um mögliche Kompatibilitätsprobleme zu identifizieren und zu beheben. Zusätzlich sollten Datenvalidierungs- und Verifizierungsprozesse implementiert werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>11442</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Die Marketingkampagnen erzielen unterdurchschnittliche Ergebnisse. Obwohl der Werbeaufwand angepasst und Inhalte aktualisiert wurden, sind die Ergebnisse immer noch unzufriedenstellend. Die uneffektiven Ziele und veralteten Inhalte könnten die Ursache sein. Wir benötigen Unterstützung, um das Problem zu lösen und die Leistung unserer Kampagnen zu verbessern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>3660</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Reklamation/Rückgabe</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Anfrage für eine sofortige Aktualisierung der Datenanalyse-Tools</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundendienst, ich möchte eine Aktualisierung unserer derzeitigen Software für Datenanalyse-Tools beantragen. Das aktuelle System ist veraltet und beeinträchtigt die Genauigkeit unserer Investitionsberichte sowie die Optimierung unserer Investitionen. Ich bitte um ein Upgrade auf die neueste Softwareversion, die Funktionen wie maschinelles Lernen und Echtzeit-Datenverarbeitung umfasst. Diese Verbesserungen würden uns helfen, fundiertere Investitionsentscheidungen zu treffen und die Gesamtleistung zu steigern. Wir würden es sehr schätzen, wenn Sie den Vorgang zeitnah prüfen und uns einen Zeitplan für die Aktualisierung mitteilen könnten. Vielen Dank für Ihre Unterstützung in dieser Angelegenheit. Ich freue mich auf Ihre baldige Rückmeldung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>23843</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>OBS Studio Integration Issue</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Beim Einbinden von OBS Studio tritt beim ClickUp ein Fehler auf. Das Problem könnte auf Kompatibilitätsprobleme beim Projektmanagement hinweisen. Software neu gestartet und Aktualisierungen überprüft, aber das Problem behält sich bestanden. Unterstützung benötigt, um das Problem zu beheben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>22319</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Preisangebote für Projektmanagement SaaS</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Geliebter Kundensupport, ich bin interessiert an weiteren Informationen zu den Preisangeboten für Projektmanagement SaaS. Könnten Sie mir detaillierte Tarife und Funktionalitäten bereitstellen? Ich möchte gerne wissen, welche Rabatte für die verschiedenen Tarife verfügbar sind. Diese Informationen könnten mir helfen, eine informierte Entscheidung zu treffen, welcher Tarif am besten für mein Geschäft geeignet ist. Vielen Dank für Ihre Unterstützung und ich freue mich auf Ihre Antwort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>14048</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr"/>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Sehr geehrte Kundensupport, ich möchte mich kontaktieren, um Informationen zu erhalten, wie ich die Datenanalysetools auf der IBM Cloud optimal nutzen kann, um meine Investitionen zu optimieren. Ich würde gerne Details über die Werkzeuge erhalten, um effektiver mit ihnen umgehen zu können und gezielte Investitionsentscheidungen treffen zu können. Ich bin sehr interessiert, mehr über die angebotenen Datenanalysetools zu erfahren, um meine Fähigkeiten in der Analyse von Marktentwicklungen, Vorhersagen für Investitionsresultate und der Erkennung von potenziellen Chancen zu verbessern. Ich freue mich darauf, Rat und Ressourcen zu erhalten. Vielen Dank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>8252</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Update der Oracle-Datenbank zur Leistungsoptimierung</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Aktualisierung der Oracle Database 19c auf Git 2.32</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>11723</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Hilfe zur digitalen Markengröße</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Könnten Sie mehr Details zu den digitalen Strategien und deren Auswirkungen auf die Markengröße geben? Ich möchte gerne mehr darüber erfahren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>24465</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Details zur Rechnungsstellung für die Airtable-Integration anfragen</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Ich bitte um weitere Informationen zur Rechnungsstellung für die Airtable-Integration im Rahmen des Projektmanagement-Software-Entwicklungsprojekts. Es wäre schön, wenn Sie mir Details zu den Preisen und möglichen Rabatten geben könnten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>5664</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Integrationsprobleme</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte auf Probleme bei der Integration digitaler Werkzeuge hinweisen, die Störungen in Marketingkampagnen verursachen. Trotz erster Maßnahmen zur Fehlerbehebung, inklusive Neustart der Anwendungen und Überprüfung der Konfigurationen, treten weiterhin Synchronisationsfehler und intermittierende Ausfälle auf. Diese Probleme beeinträchtigen die Abläufe der Kampagnen, die Genauigkeit der Analysen sowie verursachen Verzögerungen und Ineffizienzen. Ich habe versucht, das Problem durch Software-Updates zu beheben und sicherzustellen, dass die Werkzeuge kompatibel sind, doch die Schwierigkeiten bestehen weiterhin. Für Unterstützung würde ich mich sehr freuen und bitte um eine schnelle Bearbeitung der Angelegenheit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>17556</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Können Sie bitte mehr Details zu Datenanalysediensten, Optimierung und Anlageninvestitionen geben? Ich danke Ihnen für Ihre Zeit und Unterstützung bei dieser Angelegenheit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>2289</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Anfrage bezüglich Sicherheitsvorfalls in den IT-Systemen des Krankenhauses</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte einen kürzlich aufgetretenen Sicherheitsvorfall in den IT-Systemen unseres Krankenhauses melden. Es wurde festgestellt, dass Patientendaten möglicherweise aufgrund veralteter PostgreSQL-Konfigurationen offengelegt wurden. Erste Maßnahmen wie Firewall-Updates und Antiviren-Scans wurden bereits durchgeführt, doch die Schwachstellen sind weiterhin vorhanden. Zudem wurden Untersuchungen an den Integrationen der Smart-Wassermelder und der Smart-Türklingel unternommen, jedoch konnten keine Verbesserungen erzielt werden. Dieser Vorfall hat erhebliche Sicherheitsbedenken aufgeworfen, und wir sind bestrebt, eine Lösung zu finden. Für Unterstützung und eine Anleitung durch das Team wären wir dankbar, um das Problem zu beheben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>23260</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Technischer Support</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Kundenservice</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Vergrößerung</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Ich schlage vor, Verbesserungen an den Datenanalysewerkzeugen zu betreiben, um die Investitions-Optimierung, Entscheidungsfindung und Effizienz zu verbessern. Ich glaube, dass unsere aktuellen Tools nicht ausreichend sind und dass wir fortgeschrittene Funktionen wie Vorhersageanalyse und Maschinelles Lernen sehen könnten, um Muster und Trends in den Daten zu identifizieren. Zudem würde ich mehr anpassbare Dashboards und Berichte wünschen, um die individuellen Bedürfnisse der Nutzer besser zu erfüllen. Ich glaube, dass solche Verbesserungen die Effizienz der Datenanalysewerkzeuge erheblich erhöhen könnten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>23484</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Preisgestaltung für Kubernetes-Integration</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Könnten Sie die Details zu den Preisstufen für die Kubernetes-Integration liefern?</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>8647</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Rechnung/Zahlung</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Vertriebsanfrage</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Support for Drupal Commerce</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Sehr geehrter Kundenservice, ich möchte mich nach detaillierten Abrechnungs- und Zahlungsoptionen für die Integration der Drupal Commerce SaaS-Plattform erkundigen. Könnten Sie bitte weitere Informationen zu verfügbaren Zahlungsmethoden, Abonnementplänen und eventuellen zusätzlichen Gebühren im Zusammenhang mit der Integration bereitstellen? Ich würde auch gerne wissen, ob Sie Dokumentationen oder Anleitungen zur Einrichtung und Integration bereitstellen können. Vielen Dank im Voraus für Ihre Unterstützung. Ich freue mich auf Ihre baldige Rückmeldung.</t>
         </is>
       </c>
     </row>

</xml_diff>